<commit_message>
Update schema, drop all NotOntologize
</commit_message>
<xml_diff>
--- a/Excel for reference/BattINFO_converter_standard_Excel_version_1.1.17_empty.xlsx
+++ b/Excel for reference/BattINFO_converter_standard_Excel_version_1.1.17_empty.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\battinfoconverter\Excel for reference\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01AA420C-455B-4972-9AA5-ADD5D46552FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C5113F5C-C60B-4434-9E80-5594AAD21078}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="25695" yWindow="0" windowWidth="26010" windowHeight="20985" xr2:uid="{1A6D523C-FE67-4F3F-AA9B-E9FEE83DA8F2}"/>
+    <workbookView xWindow="19200" yWindow="3945" windowWidth="24060" windowHeight="16140" xr2:uid="{1A6D523C-FE67-4F3F-AA9B-E9FEE83DA8F2}"/>
   </bookViews>
   <sheets>
     <sheet name="@Schema" sheetId="2" r:id="rId1"/>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="719" uniqueCount="410">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="709" uniqueCount="415">
   <si>
     <t>Metadata</t>
   </si>
@@ -79,9 +79,6 @@
     <t>required</t>
   </si>
   <si>
-    <t>NotOntologize</t>
-  </si>
-  <si>
     <t>Cell ID</t>
   </si>
   <si>
@@ -1243,9 +1240,6 @@
     <t>empa__ccid_123456</t>
   </si>
   <si>
-    <t>REQUIRED, CANNOT BE CHANGED. Unique ID for cell.</t>
-  </si>
-  <si>
     <t>Cell label</t>
   </si>
   <si>
@@ -1255,9 +1249,6 @@
     <t>Human-friendly name or label for cell</t>
   </si>
   <si>
-    <t>REQUIRED, CANNOT BE CHANGED. Value should be in @classes with ID</t>
-  </si>
-  <si>
     <t>Battery2030+/PREMISE</t>
   </si>
   <si>
@@ -1273,7 +1264,31 @@
     <t>240616_bco_gr-NMC_01</t>
   </si>
   <si>
-    <t>REQUIRED, CANNOT BE CHANGED. Assembly date in ISO8601 format (YYYY-MM-DD).</t>
+    <t>type|</t>
+  </si>
+  <si>
+    <t>schema:productID</t>
+  </si>
+  <si>
+    <t>schema:dateCreated</t>
+  </si>
+  <si>
+    <t>schema:manufacturer</t>
+  </si>
+  <si>
+    <t>schema:creator</t>
+  </si>
+  <si>
+    <t>rdfs:comment</t>
+  </si>
+  <si>
+    <t>REQUIRED, CANNOT BE CHANGED, unique ID for cell</t>
+  </si>
+  <si>
+    <t>REQUIRED, CANNOT BE CHANGED, assembly date in ISO8601 format (YYYY-MM-DD)</t>
+  </si>
+  <si>
+    <t>REQUIRED, CANNOT BE CHANGED, value should be in @classes with ID</t>
   </si>
 </sst>
 </file>
@@ -1282,7 +1297,7 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
     <numFmt numFmtId="164" formatCode="0.0"/>
-    <numFmt numFmtId="166" formatCode="yyyy\-mm\-dd;@"/>
+    <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd;@"/>
   </numFmts>
   <fonts count="13">
     <font>
@@ -1658,7 +1673,7 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="4" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="4" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2406,18 +2421,18 @@
         <v>10</v>
       </c>
       <c r="E3" s="13" t="s">
-        <v>11</v>
+        <v>406</v>
       </c>
       <c r="F3" s="13" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="15" customHeight="1" outlineLevel="1">
       <c r="A4" s="14" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B4" s="40" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="C4" s="14" t="s">
         <v>9</v>
@@ -2426,35 +2441,35 @@
         <v>10</v>
       </c>
       <c r="E4" s="14" t="s">
-        <v>11</v>
+        <v>407</v>
       </c>
       <c r="F4" s="14" t="s">
-        <v>399</v>
+        <v>412</v>
       </c>
     </row>
     <row r="5" spans="1:6" outlineLevel="1">
       <c r="A5" s="13" t="s">
+        <v>398</v>
+      </c>
+      <c r="B5" s="39" t="s">
+        <v>405</v>
+      </c>
+      <c r="C5" s="13" t="s">
+        <v>9</v>
+      </c>
+      <c r="D5" s="13" t="s">
+        <v>18</v>
+      </c>
+      <c r="E5" s="13" t="s">
+        <v>399</v>
+      </c>
+      <c r="F5" s="13" t="s">
         <v>400</v>
-      </c>
-      <c r="B5" s="39" t="s">
-        <v>408</v>
-      </c>
-      <c r="C5" s="13" t="s">
-        <v>9</v>
-      </c>
-      <c r="D5" s="13" t="s">
-        <v>19</v>
-      </c>
-      <c r="E5" s="13" t="s">
-        <v>401</v>
-      </c>
-      <c r="F5" s="13" t="s">
-        <v>402</v>
       </c>
     </row>
     <row r="6" spans="1:6" outlineLevel="1">
       <c r="A6" s="14" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B6" s="66">
         <v>45459</v>
@@ -2466,18 +2481,18 @@
         <v>10</v>
       </c>
       <c r="E6" s="14" t="s">
-        <v>11</v>
+        <v>408</v>
       </c>
       <c r="F6" s="14" t="s">
-        <v>409</v>
+        <v>413</v>
       </c>
     </row>
     <row r="7" spans="1:6" outlineLevel="1">
       <c r="A7" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="B7" s="39" t="s">
         <v>14</v>
-      </c>
-      <c r="B7" s="39" t="s">
-        <v>15</v>
       </c>
       <c r="C7" s="13" t="s">
         <v>9</v>
@@ -2486,18 +2501,18 @@
         <v>10</v>
       </c>
       <c r="E7" s="13" t="s">
-        <v>11</v>
-      </c>
-      <c r="F7" s="14" t="s">
-        <v>403</v>
+        <v>409</v>
+      </c>
+      <c r="F7" s="13" t="s">
+        <v>414</v>
       </c>
     </row>
     <row r="8" spans="1:6" outlineLevel="1">
       <c r="A8" s="14" t="s">
+        <v>15</v>
+      </c>
+      <c r="B8" s="40" t="s">
         <v>16</v>
-      </c>
-      <c r="B8" s="40" t="s">
-        <v>17</v>
       </c>
       <c r="C8" s="14" t="s">
         <v>9</v>
@@ -2506,54 +2521,54 @@
         <v>10</v>
       </c>
       <c r="E8" s="14" t="s">
-        <v>11</v>
+        <v>410</v>
       </c>
       <c r="F8" s="14" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
     </row>
     <row r="9" spans="1:6" outlineLevel="1">
       <c r="A9" s="13" t="s">
+        <v>17</v>
+      </c>
+      <c r="B9" s="39" t="s">
+        <v>401</v>
+      </c>
+      <c r="C9" s="13" t="s">
+        <v>9</v>
+      </c>
+      <c r="D9" s="13" t="s">
         <v>18</v>
       </c>
-      <c r="B9" s="39" t="s">
-        <v>404</v>
-      </c>
-      <c r="C9" s="13" t="s">
-        <v>9</v>
-      </c>
-      <c r="D9" s="13" t="s">
-        <v>19</v>
-      </c>
       <c r="E9" s="13" t="s">
-        <v>5</v>
+        <v>411</v>
       </c>
       <c r="F9" s="13"/>
     </row>
     <row r="10" spans="1:6" outlineLevel="1">
       <c r="A10" s="14" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B10" s="40" t="s">
-        <v>405</v>
+        <v>402</v>
       </c>
       <c r="C10" s="14" t="s">
         <v>9</v>
       </c>
       <c r="D10" s="14" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E10" s="14" t="s">
-        <v>5</v>
+        <v>411</v>
       </c>
       <c r="F10" s="14"/>
     </row>
     <row r="11" spans="1:6" outlineLevel="1">
       <c r="A11" s="13" t="s">
+        <v>388</v>
+      </c>
+      <c r="B11" s="39" t="s">
         <v>389</v>
-      </c>
-      <c r="B11" s="39" t="s">
-        <v>390</v>
       </c>
       <c r="C11" s="13" t="s">
         <v>9</v>
@@ -2562,18 +2577,18 @@
         <v>10</v>
       </c>
       <c r="E11" s="13" t="s">
-        <v>5</v>
+        <v>411</v>
       </c>
       <c r="F11" s="13" t="s">
-        <v>406</v>
+        <v>403</v>
       </c>
     </row>
     <row r="12" spans="1:6" outlineLevel="1">
       <c r="A12" s="14" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="B12" s="40" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="C12" s="14" t="s">
         <v>9</v>
@@ -2582,15 +2597,15 @@
         <v>10</v>
       </c>
       <c r="E12" s="14" t="s">
-        <v>5</v>
+        <v>411</v>
       </c>
       <c r="F12" s="14" t="s">
-        <v>407</v>
+        <v>404</v>
       </c>
     </row>
     <row r="13" spans="1:6">
       <c r="A13" s="30" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B13" s="41"/>
       <c r="C13" s="15"/>
@@ -2600,7 +2615,7 @@
     </row>
     <row r="14" spans="1:6" outlineLevel="1">
       <c r="A14" s="13" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B14" s="39"/>
       <c r="C14" s="13" t="s">
@@ -2610,29 +2625,29 @@
         <v>10</v>
       </c>
       <c r="E14" s="13" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F14" s="13"/>
     </row>
     <row r="15" spans="1:6" outlineLevel="1">
       <c r="A15" s="16" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B15" s="42"/>
       <c r="C15" s="16" t="s">
+        <v>25</v>
+      </c>
+      <c r="D15" s="16" t="s">
+        <v>18</v>
+      </c>
+      <c r="E15" s="16" t="s">
         <v>26</v>
-      </c>
-      <c r="D15" s="16" t="s">
-        <v>19</v>
-      </c>
-      <c r="E15" s="16" t="s">
-        <v>27</v>
       </c>
       <c r="F15" s="16"/>
     </row>
     <row r="16" spans="1:6" outlineLevel="1">
       <c r="A16" s="13" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B16" s="39"/>
       <c r="C16" s="13" t="s">
@@ -2642,45 +2657,45 @@
         <v>10</v>
       </c>
       <c r="E16" s="13" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F16" s="13"/>
     </row>
     <row r="17" spans="1:6" outlineLevel="1">
       <c r="A17" s="16" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B17" s="42"/>
       <c r="C17" s="16" t="s">
         <v>9</v>
       </c>
       <c r="D17" s="16" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E17" s="16" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="F17" s="16"/>
     </row>
     <row r="18" spans="1:6" outlineLevel="1">
       <c r="A18" s="13" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B18" s="39"/>
       <c r="C18" s="13" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D18" s="13" t="s">
         <v>10</v>
       </c>
       <c r="E18" s="13" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="F18" s="13"/>
     </row>
     <row r="19" spans="1:6" outlineLevel="1">
       <c r="A19" s="16" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B19" s="42"/>
       <c r="C19" s="16" t="s">
@@ -2690,29 +2705,29 @@
         <v>10</v>
       </c>
       <c r="E19" s="16" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="F19" s="16"/>
     </row>
     <row r="20" spans="1:6" outlineLevel="1">
       <c r="A20" s="13" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B20" s="39"/>
       <c r="C20" s="13" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D20" s="13" t="s">
         <v>10</v>
       </c>
       <c r="E20" s="13" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="F20" s="13"/>
     </row>
     <row r="21" spans="1:6" ht="15.75" customHeight="1" outlineLevel="1">
       <c r="A21" s="16" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B21" s="42"/>
       <c r="C21" s="16" t="s">
@@ -2722,513 +2737,507 @@
         <v>10</v>
       </c>
       <c r="E21" s="16" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F21" s="16"/>
     </row>
     <row r="22" spans="1:6" outlineLevel="1">
       <c r="A22" s="13" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B22" s="39"/>
       <c r="C22" s="13" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D22" s="13" t="s">
         <v>10</v>
       </c>
       <c r="E22" s="13" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="F22" s="13"/>
     </row>
     <row r="23" spans="1:6" outlineLevel="1">
       <c r="A23" s="16" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B23" s="42"/>
       <c r="C23" s="16" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D23" s="16" t="s">
         <v>10</v>
       </c>
       <c r="E23" s="16" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="F23" s="16"/>
     </row>
     <row r="24" spans="1:6" outlineLevel="1">
       <c r="A24" s="13" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B24" s="39"/>
       <c r="C24" s="13" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D24" s="13" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E24" s="13" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="F24" s="13"/>
     </row>
     <row r="25" spans="1:6">
       <c r="A25" s="31" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B25" s="43"/>
       <c r="C25" s="15"/>
       <c r="D25" s="15"/>
-      <c r="E25" s="15" t="s">
-        <v>11</v>
-      </c>
+      <c r="E25" s="15"/>
       <c r="F25" s="15"/>
     </row>
     <row r="26" spans="1:6" outlineLevel="1">
       <c r="A26" s="13" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B26" s="39"/>
       <c r="C26" s="13" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D26" s="13" t="s">
+        <v>50</v>
+      </c>
+      <c r="E26" s="13" t="s">
         <v>51</v>
-      </c>
-      <c r="E26" s="13" t="s">
-        <v>52</v>
       </c>
       <c r="F26" s="13"/>
     </row>
     <row r="27" spans="1:6" outlineLevel="1">
       <c r="A27" s="16" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B27" s="44"/>
       <c r="C27" s="16" t="s">
+        <v>53</v>
+      </c>
+      <c r="D27" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="E27" s="16" t="s">
         <v>54</v>
-      </c>
-      <c r="D27" s="16" t="s">
-        <v>51</v>
-      </c>
-      <c r="E27" s="16" t="s">
-        <v>55</v>
       </c>
       <c r="F27" s="16"/>
     </row>
     <row r="28" spans="1:6" outlineLevel="1">
       <c r="A28" s="13" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B28" s="39"/>
       <c r="C28" s="13" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D28" s="13" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E28" s="13" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="F28" s="13"/>
     </row>
     <row r="29" spans="1:6">
       <c r="A29" s="31" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B29" s="43"/>
       <c r="C29" s="15"/>
       <c r="D29" s="15"/>
-      <c r="E29" s="15" t="s">
-        <v>11</v>
-      </c>
+      <c r="E29" s="15"/>
       <c r="F29" s="15"/>
     </row>
     <row r="30" spans="1:6" outlineLevel="1">
       <c r="A30" s="13" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B30" s="39"/>
       <c r="C30" s="13" t="s">
         <v>9</v>
       </c>
       <c r="D30" s="13" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E30" s="13" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="F30" s="13"/>
     </row>
     <row r="31" spans="1:6" outlineLevel="1">
       <c r="A31" s="16" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B31" s="42"/>
       <c r="C31" s="16" t="s">
         <v>9</v>
       </c>
       <c r="D31" s="16" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E31" s="16" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="F31" s="16"/>
     </row>
     <row r="32" spans="1:6" outlineLevel="1">
       <c r="A32" s="13" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B32" s="45"/>
       <c r="C32" s="13" t="s">
+        <v>64</v>
+      </c>
+      <c r="D32" s="13" t="s">
+        <v>50</v>
+      </c>
+      <c r="E32" s="13" t="s">
         <v>65</v>
-      </c>
-      <c r="D32" s="13" t="s">
-        <v>51</v>
-      </c>
-      <c r="E32" s="13" t="s">
-        <v>66</v>
       </c>
       <c r="F32" s="13"/>
     </row>
     <row r="33" spans="1:6" outlineLevel="1">
       <c r="A33" s="16" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B33" s="42"/>
       <c r="C33" s="16" t="s">
+        <v>67</v>
+      </c>
+      <c r="D33" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="E33" s="16" t="s">
         <v>68</v>
-      </c>
-      <c r="D33" s="16" t="s">
-        <v>51</v>
-      </c>
-      <c r="E33" s="16" t="s">
-        <v>69</v>
       </c>
       <c r="F33" s="16"/>
     </row>
     <row r="34" spans="1:6" outlineLevel="1">
       <c r="A34" s="13" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B34" s="39"/>
       <c r="C34" s="13" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D34" s="13" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E34" s="13" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="F34" s="13"/>
     </row>
     <row r="35" spans="1:6" outlineLevel="1">
       <c r="A35" s="16" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B35" s="42"/>
       <c r="C35" s="16" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D35" s="16" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E35" s="16" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="F35" s="16"/>
     </row>
     <row r="36" spans="1:6" outlineLevel="1">
       <c r="A36" s="13" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B36" s="39"/>
       <c r="C36" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D36" s="13" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E36" s="13" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="F36" s="13"/>
     </row>
     <row r="37" spans="1:6" outlineLevel="1">
       <c r="A37" s="16" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B37" s="42"/>
       <c r="C37" s="16" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D37" s="16" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E37" s="16" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="F37" s="16"/>
     </row>
     <row r="38" spans="1:6" outlineLevel="1">
       <c r="A38" s="13" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B38" s="46"/>
       <c r="C38" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D38" s="13" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E38" s="13" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="F38" s="13"/>
     </row>
     <row r="39" spans="1:6" outlineLevel="1">
       <c r="A39" s="16" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B39" s="42"/>
       <c r="C39" s="16" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D39" s="16" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E39" s="16" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="F39" s="16"/>
     </row>
     <row r="40" spans="1:6" outlineLevel="1">
       <c r="A40" s="13" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B40" s="45"/>
       <c r="C40" s="13" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D40" s="13" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E40" s="13" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="F40" s="13"/>
     </row>
     <row r="41" spans="1:6" outlineLevel="1">
       <c r="A41" s="16" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B41" s="47"/>
       <c r="C41" s="16" t="s">
+        <v>84</v>
+      </c>
+      <c r="D41" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="E41" s="16" t="s">
         <v>85</v>
-      </c>
-      <c r="D41" s="16" t="s">
-        <v>51</v>
-      </c>
-      <c r="E41" s="16" t="s">
-        <v>86</v>
       </c>
       <c r="F41" s="16"/>
     </row>
     <row r="42" spans="1:6" outlineLevel="1">
       <c r="A42" s="13" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B42" s="39"/>
       <c r="C42" s="13" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D42" s="13" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E42" s="13" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="F42" s="13"/>
     </row>
     <row r="43" spans="1:6">
       <c r="A43" s="31" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B43" s="43"/>
       <c r="C43" s="15"/>
       <c r="D43" s="15"/>
-      <c r="E43" s="15" t="s">
-        <v>11</v>
-      </c>
+      <c r="E43" s="15"/>
       <c r="F43" s="15"/>
     </row>
     <row r="44" spans="1:6" outlineLevel="1">
       <c r="A44" s="13" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B44" s="39"/>
       <c r="C44" s="13" t="s">
         <v>9</v>
       </c>
       <c r="D44" s="13" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E44" s="13" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="F44" s="13"/>
     </row>
     <row r="45" spans="1:6" outlineLevel="1">
       <c r="A45" s="16" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B45" s="42"/>
       <c r="C45" s="16" t="s">
         <v>9</v>
       </c>
       <c r="D45" s="16" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E45" s="16" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="F45" s="16"/>
     </row>
     <row r="46" spans="1:6" outlineLevel="1">
       <c r="A46" s="13" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B46" s="39"/>
       <c r="C46" s="13" t="s">
         <v>9</v>
       </c>
       <c r="D46" s="13" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E46" s="13" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="F46" s="13"/>
     </row>
     <row r="47" spans="1:6" outlineLevel="1">
       <c r="A47" s="16" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B47" s="42"/>
       <c r="C47" s="16" t="s">
         <v>9</v>
       </c>
       <c r="D47" s="16" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E47" s="16" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="F47" s="16"/>
     </row>
     <row r="48" spans="1:6" outlineLevel="1">
       <c r="A48" s="13" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B48" s="39"/>
       <c r="C48" s="13" t="s">
         <v>9</v>
       </c>
       <c r="D48" s="13" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E48" s="13" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="F48" s="13"/>
     </row>
     <row r="49" spans="1:6" outlineLevel="1">
       <c r="A49" s="16" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B49" s="42"/>
       <c r="C49" s="16" t="s">
         <v>9</v>
       </c>
       <c r="D49" s="16" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E49" s="16" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="F49" s="16"/>
     </row>
     <row r="50" spans="1:6" outlineLevel="1">
       <c r="A50" s="13" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B50" s="39"/>
       <c r="C50" s="13" t="s">
         <v>9</v>
       </c>
       <c r="D50" s="13" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E50" s="13" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="F50" s="13"/>
     </row>
     <row r="51" spans="1:6" outlineLevel="1">
       <c r="A51" s="16" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B51" s="42"/>
       <c r="C51" s="16" t="s">
         <v>9</v>
       </c>
       <c r="D51" s="16" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E51" s="16" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="F51" s="16"/>
     </row>
     <row r="52" spans="1:6" outlineLevel="1">
       <c r="A52" s="13" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B52" s="39"/>
       <c r="C52" s="13" t="s">
         <v>9</v>
       </c>
       <c r="D52" s="13" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E52" s="13" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="F52" s="13"/>
     </row>
     <row r="53" spans="1:6" outlineLevel="1">
       <c r="A53" s="16" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B53" s="42"/>
       <c r="C53" s="16" t="s">
         <v>9</v>
       </c>
       <c r="D53" s="16" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E53" s="16" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="F53" s="16"/>
     </row>
     <row r="54" spans="1:6">
       <c r="A54" s="32" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B54" s="48"/>
       <c r="C54" s="17"/>
@@ -3238,7 +3247,7 @@
     </row>
     <row r="55" spans="1:6" outlineLevel="1">
       <c r="A55" s="18" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B55" s="49"/>
       <c r="C55" s="18" t="s">
@@ -3248,29 +3257,29 @@
         <v>10</v>
       </c>
       <c r="E55" s="18" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="F55" s="18"/>
     </row>
     <row r="56" spans="1:6" outlineLevel="1">
       <c r="A56" s="13" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B56" s="39"/>
       <c r="C56" s="13" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D56" s="13" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E56" s="13" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="F56" s="13"/>
     </row>
     <row r="57" spans="1:6" outlineLevel="1">
       <c r="A57" s="18" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B57" s="49"/>
       <c r="C57" s="18" t="s">
@@ -3280,29 +3289,29 @@
         <v>10</v>
       </c>
       <c r="E57" s="18" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="F57" s="18"/>
     </row>
     <row r="58" spans="1:6" outlineLevel="1">
       <c r="A58" s="13" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="B58" s="39"/>
       <c r="C58" s="13" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D58" s="13" t="s">
         <v>10</v>
       </c>
       <c r="E58" s="13" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="F58" s="13"/>
     </row>
     <row r="59" spans="1:6" outlineLevel="1">
       <c r="A59" s="18" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B59" s="49"/>
       <c r="C59" s="18" t="s">
@@ -3312,29 +3321,29 @@
         <v>10</v>
       </c>
       <c r="E59" s="18" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="F59" s="18"/>
     </row>
     <row r="60" spans="1:6" outlineLevel="1">
       <c r="A60" s="13" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B60" s="39"/>
       <c r="C60" s="13" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D60" s="13" t="s">
         <v>10</v>
       </c>
       <c r="E60" s="13" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F60" s="13"/>
     </row>
     <row r="61" spans="1:6" outlineLevel="1">
       <c r="A61" s="18" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B61" s="49"/>
       <c r="C61" s="18" t="s">
@@ -3344,513 +3353,507 @@
         <v>10</v>
       </c>
       <c r="E61" s="18" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="F61" s="18"/>
     </row>
     <row r="62" spans="1:6" outlineLevel="1">
       <c r="A62" s="13" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B62" s="39"/>
       <c r="C62" s="13" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D62" s="13" t="s">
         <v>10</v>
       </c>
       <c r="E62" s="13" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="F62" s="13"/>
     </row>
     <row r="63" spans="1:6" outlineLevel="1">
       <c r="A63" s="18" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B63" s="49"/>
       <c r="C63" s="18" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D63" s="18" t="s">
         <v>10</v>
       </c>
       <c r="E63" s="18" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="F63" s="18"/>
     </row>
     <row r="64" spans="1:6" outlineLevel="1">
       <c r="A64" s="13" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B64" s="39"/>
       <c r="C64" s="13" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D64" s="13" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E64" s="13" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="F64" s="13"/>
     </row>
     <row r="65" spans="1:6">
       <c r="A65" s="33" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="B65" s="50"/>
       <c r="C65" s="19"/>
       <c r="D65" s="19"/>
-      <c r="E65" s="19" t="s">
-        <v>11</v>
-      </c>
+      <c r="E65" s="19"/>
       <c r="F65" s="19"/>
     </row>
     <row r="66" spans="1:6" outlineLevel="1">
       <c r="A66" s="13" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B66" s="39"/>
       <c r="C66" s="13" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D66" s="13" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E66" s="13" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="F66" s="13"/>
     </row>
     <row r="67" spans="1:6" outlineLevel="1">
       <c r="A67" s="18" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B67" s="51"/>
       <c r="C67" s="18" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D67" s="18" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E67" s="18" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="F67" s="18"/>
     </row>
     <row r="68" spans="1:6" outlineLevel="1">
       <c r="A68" s="13" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B68" s="39"/>
       <c r="C68" s="13" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D68" s="13" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E68" s="13" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="F68" s="13"/>
     </row>
     <row r="69" spans="1:6">
       <c r="A69" s="33" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B69" s="50"/>
       <c r="C69" s="19"/>
       <c r="D69" s="19"/>
-      <c r="E69" s="19" t="s">
-        <v>11</v>
-      </c>
+      <c r="E69" s="19"/>
       <c r="F69" s="19"/>
     </row>
     <row r="70" spans="1:6" outlineLevel="1">
       <c r="A70" s="13" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="B70" s="39"/>
       <c r="C70" s="13" t="s">
         <v>9</v>
       </c>
       <c r="D70" s="13" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E70" s="13" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="F70" s="13"/>
     </row>
     <row r="71" spans="1:6" outlineLevel="1">
       <c r="A71" s="18" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B71" s="52"/>
       <c r="C71" s="18" t="s">
         <v>9</v>
       </c>
       <c r="D71" s="18" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E71" s="18" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="F71" s="18"/>
     </row>
     <row r="72" spans="1:6" outlineLevel="1">
       <c r="A72" s="13" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B72" s="46"/>
       <c r="C72" s="13" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D72" s="13" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E72" s="13" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="F72" s="13"/>
     </row>
     <row r="73" spans="1:6" outlineLevel="1">
       <c r="A73" s="18" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B73" s="53"/>
       <c r="C73" s="18" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D73" s="18" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E73" s="18" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="F73" s="18"/>
     </row>
     <row r="74" spans="1:6" outlineLevel="1">
       <c r="A74" s="13" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B74" s="39"/>
       <c r="C74" s="13" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D74" s="13" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E74" s="13" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="F74" s="13"/>
     </row>
     <row r="75" spans="1:6" outlineLevel="1">
       <c r="A75" s="18" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B75" s="53"/>
       <c r="C75" s="18" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D75" s="18" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E75" s="18" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="F75" s="18"/>
     </row>
     <row r="76" spans="1:6" outlineLevel="1">
       <c r="A76" s="13" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B76" s="39"/>
       <c r="C76" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D76" s="13" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E76" s="13" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="F76" s="13"/>
     </row>
     <row r="77" spans="1:6" outlineLevel="1">
       <c r="A77" s="18" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B77" s="53"/>
       <c r="C77" s="18" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D77" s="18" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E77" s="18" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="F77" s="18"/>
     </row>
     <row r="78" spans="1:6" outlineLevel="1">
       <c r="A78" s="13" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B78" s="46"/>
       <c r="C78" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D78" s="13" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E78" s="13" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="F78" s="13"/>
     </row>
     <row r="79" spans="1:6" outlineLevel="1">
       <c r="A79" s="18" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B79" s="53"/>
       <c r="C79" s="18" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D79" s="18" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E79" s="18" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="F79" s="18"/>
     </row>
     <row r="80" spans="1:6" outlineLevel="1">
       <c r="A80" s="13" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B80" s="46"/>
       <c r="C80" s="13" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D80" s="13" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E80" s="13" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="F80" s="13"/>
     </row>
     <row r="81" spans="1:6" outlineLevel="1">
       <c r="A81" s="18" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="B81" s="54"/>
       <c r="C81" s="18" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D81" s="18" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E81" s="18" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="F81" s="18"/>
     </row>
     <row r="82" spans="1:6" outlineLevel="1">
       <c r="A82" s="13" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="B82" s="55"/>
       <c r="C82" s="13" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D82" s="13" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E82" s="13" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="F82" s="13"/>
     </row>
     <row r="83" spans="1:6">
       <c r="A83" s="33" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="B83" s="50"/>
       <c r="C83" s="19"/>
       <c r="D83" s="19"/>
-      <c r="E83" s="19" t="s">
-        <v>11</v>
-      </c>
+      <c r="E83" s="19"/>
       <c r="F83" s="19"/>
     </row>
     <row r="84" spans="1:6" outlineLevel="1">
       <c r="A84" s="13" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="B84" s="39"/>
       <c r="C84" s="13" t="s">
         <v>9</v>
       </c>
       <c r="D84" s="13" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E84" s="13" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="F84" s="13"/>
     </row>
     <row r="85" spans="1:6" outlineLevel="1">
       <c r="A85" s="18" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="B85" s="49"/>
       <c r="C85" s="18" t="s">
         <v>9</v>
       </c>
       <c r="D85" s="18" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E85" s="18" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="F85" s="18"/>
     </row>
     <row r="86" spans="1:6" outlineLevel="1">
       <c r="A86" s="13" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B86" s="39"/>
       <c r="C86" s="13" t="s">
         <v>9</v>
       </c>
       <c r="D86" s="13" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E86" s="13" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="F86" s="13"/>
     </row>
     <row r="87" spans="1:6" outlineLevel="1">
       <c r="A87" s="18" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B87" s="49"/>
       <c r="C87" s="18" t="s">
         <v>9</v>
       </c>
       <c r="D87" s="18" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E87" s="18" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="F87" s="18"/>
     </row>
     <row r="88" spans="1:6" outlineLevel="1">
       <c r="A88" s="13" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="B88" s="39"/>
       <c r="C88" s="13" t="s">
         <v>9</v>
       </c>
       <c r="D88" s="13" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E88" s="13" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="F88" s="13"/>
     </row>
     <row r="89" spans="1:6" outlineLevel="1">
       <c r="A89" s="18" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="B89" s="49"/>
       <c r="C89" s="18" t="s">
         <v>9</v>
       </c>
       <c r="D89" s="18" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E89" s="18" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="F89" s="18"/>
     </row>
     <row r="90" spans="1:6" outlineLevel="1">
       <c r="A90" s="13" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="B90" s="39"/>
       <c r="C90" s="13" t="s">
         <v>9</v>
       </c>
       <c r="D90" s="13" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E90" s="13" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="F90" s="13"/>
     </row>
     <row r="91" spans="1:6" outlineLevel="1">
       <c r="A91" s="18" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="B91" s="49"/>
       <c r="C91" s="18" t="s">
         <v>9</v>
       </c>
       <c r="D91" s="18" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E91" s="18" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="F91" s="18"/>
     </row>
     <row r="92" spans="1:6" outlineLevel="1">
       <c r="A92" s="13" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="B92" s="39"/>
       <c r="C92" s="13" t="s">
         <v>9</v>
       </c>
       <c r="D92" s="13" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E92" s="13" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="F92" s="13"/>
     </row>
     <row r="93" spans="1:6" outlineLevel="1">
       <c r="A93" s="18" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="B93" s="49"/>
       <c r="C93" s="18" t="s">
         <v>9</v>
       </c>
       <c r="D93" s="18" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E93" s="18" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="F93" s="18"/>
     </row>
     <row r="94" spans="1:6">
       <c r="A94" s="34" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="B94" s="56"/>
       <c r="C94" s="20"/>
@@ -3860,7 +3863,7 @@
     </row>
     <row r="95" spans="1:6" outlineLevel="1">
       <c r="A95" s="13" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="B95" s="39"/>
       <c r="C95" s="13" t="s">
@@ -3870,61 +3873,61 @@
         <v>10</v>
       </c>
       <c r="E95" s="13" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="F95" s="13"/>
     </row>
     <row r="96" spans="1:6" outlineLevel="1">
       <c r="A96" s="21" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="B96" s="57"/>
       <c r="C96" s="21" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D96" s="21" t="s">
         <v>10</v>
       </c>
       <c r="E96" s="21" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="F96" s="21"/>
     </row>
     <row r="97" spans="1:6" outlineLevel="1">
       <c r="A97" s="13" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="B97" s="39"/>
       <c r="C97" s="13" t="s">
         <v>9</v>
       </c>
       <c r="D97" s="13" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E97" s="13" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="F97" s="13"/>
     </row>
     <row r="98" spans="1:6" outlineLevel="1">
       <c r="A98" s="21" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="B98" s="57"/>
       <c r="C98" s="21" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D98" s="22" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E98" s="21" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="F98" s="21"/>
     </row>
     <row r="99" spans="1:6" outlineLevel="1">
       <c r="A99" s="13" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="B99" s="39"/>
       <c r="C99" s="13" t="s">
@@ -3934,437 +3937,433 @@
         <v>10</v>
       </c>
       <c r="E99" s="13" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="F99" s="13"/>
     </row>
     <row r="100" spans="1:6" outlineLevel="1">
       <c r="A100" s="21" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="B100" s="57"/>
       <c r="C100" s="21" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="D100" s="21" t="s">
         <v>10</v>
       </c>
       <c r="E100" s="21" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="F100" s="21"/>
     </row>
     <row r="101" spans="1:6" outlineLevel="1">
       <c r="A101" s="13" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="B101" s="39"/>
       <c r="C101" s="13" t="s">
         <v>9</v>
       </c>
       <c r="D101" s="13" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E101" s="13" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="F101" s="13"/>
     </row>
     <row r="102" spans="1:6" outlineLevel="1">
       <c r="A102" s="21" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B102" s="57"/>
       <c r="C102" s="21" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="D102" s="21" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E102" s="21" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="F102" s="21"/>
     </row>
     <row r="103" spans="1:6" outlineLevel="1">
       <c r="A103" s="13" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="B103" s="39"/>
       <c r="C103" s="13" t="s">
         <v>9</v>
       </c>
       <c r="D103" s="13" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E103" s="13" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="F103" s="13"/>
     </row>
     <row r="104" spans="1:6" outlineLevel="1">
       <c r="A104" s="21" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="B104" s="57"/>
       <c r="C104" s="21" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="D104" s="21" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E104" s="21" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="F104" s="21"/>
     </row>
     <row r="105" spans="1:6" outlineLevel="1">
       <c r="A105" s="13" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="B105" s="39"/>
       <c r="C105" s="13" t="s">
         <v>9</v>
       </c>
       <c r="D105" s="13" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E105" s="13" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="F105" s="13"/>
     </row>
     <row r="106" spans="1:6" outlineLevel="1">
       <c r="A106" s="21" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B106" s="57"/>
       <c r="C106" s="21" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="D106" s="21" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E106" s="21" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="F106" s="21"/>
     </row>
     <row r="107" spans="1:6">
       <c r="A107" s="35" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B107" s="58"/>
       <c r="C107" s="20"/>
       <c r="D107" s="20"/>
-      <c r="E107" s="20" t="s">
-        <v>11</v>
-      </c>
+      <c r="E107" s="20"/>
       <c r="F107" s="20"/>
     </row>
     <row r="108" spans="1:6" outlineLevel="1">
       <c r="A108" s="21" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B108" s="57"/>
       <c r="C108" s="21" t="s">
+        <v>197</v>
+      </c>
+      <c r="D108" s="21" t="s">
+        <v>50</v>
+      </c>
+      <c r="E108" s="21" t="s">
         <v>198</v>
-      </c>
-      <c r="D108" s="21" t="s">
-        <v>51</v>
-      </c>
-      <c r="E108" s="21" t="s">
-        <v>199</v>
       </c>
       <c r="F108" s="21"/>
     </row>
     <row r="109" spans="1:6" outlineLevel="1">
       <c r="A109" s="13" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="B109" s="59"/>
       <c r="C109" s="13" t="s">
+        <v>200</v>
+      </c>
+      <c r="D109" s="13" t="s">
+        <v>50</v>
+      </c>
+      <c r="E109" s="13" t="s">
         <v>201</v>
-      </c>
-      <c r="D109" s="13" t="s">
-        <v>51</v>
-      </c>
-      <c r="E109" s="13" t="s">
-        <v>202</v>
       </c>
       <c r="F109" s="13"/>
     </row>
     <row r="110" spans="1:6" outlineLevel="1">
       <c r="A110" s="21" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="B110" s="57"/>
       <c r="C110" s="21" t="s">
+        <v>203</v>
+      </c>
+      <c r="D110" s="21" t="s">
+        <v>50</v>
+      </c>
+      <c r="E110" s="21" t="s">
         <v>204</v>
-      </c>
-      <c r="D110" s="21" t="s">
-        <v>51</v>
-      </c>
-      <c r="E110" s="21" t="s">
-        <v>205</v>
       </c>
       <c r="F110" s="21"/>
     </row>
     <row r="111" spans="1:6" outlineLevel="1">
       <c r="A111" s="13" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="B111" s="59"/>
       <c r="C111" s="13" t="s">
+        <v>206</v>
+      </c>
+      <c r="D111" s="13" t="s">
+        <v>50</v>
+      </c>
+      <c r="E111" s="23" t="s">
         <v>207</v>
-      </c>
-      <c r="D111" s="13" t="s">
-        <v>51</v>
-      </c>
-      <c r="E111" s="23" t="s">
-        <v>208</v>
       </c>
       <c r="F111" s="13"/>
     </row>
     <row r="112" spans="1:6">
       <c r="A112" s="35" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="B112" s="58"/>
       <c r="C112" s="20"/>
       <c r="D112" s="20"/>
-      <c r="E112" s="20" t="s">
-        <v>11</v>
-      </c>
+      <c r="E112" s="20"/>
       <c r="F112" s="20"/>
     </row>
     <row r="113" spans="1:6" outlineLevel="1">
       <c r="A113" s="13" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B113" s="39"/>
       <c r="C113" s="13" t="s">
         <v>9</v>
       </c>
       <c r="D113" s="13" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E113" s="13" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="F113" s="13"/>
     </row>
     <row r="114" spans="1:6" outlineLevel="1">
       <c r="A114" s="21" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="B114" s="57"/>
       <c r="C114" s="21" t="s">
         <v>9</v>
       </c>
       <c r="D114" s="21" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E114" s="21" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="F114" s="21"/>
     </row>
     <row r="115" spans="1:6" outlineLevel="1">
       <c r="A115" s="13" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="B115" s="39"/>
       <c r="C115" s="13" t="s">
         <v>9</v>
       </c>
       <c r="D115" s="13" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E115" s="13" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="F115" s="13"/>
     </row>
     <row r="116" spans="1:6" outlineLevel="1">
       <c r="A116" s="21" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="B116" s="57"/>
       <c r="C116" s="21" t="s">
         <v>9</v>
       </c>
       <c r="D116" s="21" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E116" s="21" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="F116" s="21"/>
     </row>
     <row r="117" spans="1:6" outlineLevel="1">
       <c r="A117" s="13" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="B117" s="39"/>
       <c r="C117" s="13" t="s">
         <v>9</v>
       </c>
       <c r="D117" s="13" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E117" s="13" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="F117" s="13"/>
     </row>
     <row r="118" spans="1:6" outlineLevel="1">
       <c r="A118" s="24" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="B118" s="60"/>
       <c r="C118" s="24" t="s">
         <v>9</v>
       </c>
       <c r="D118" s="24" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E118" s="24" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="F118" s="21"/>
     </row>
     <row r="119" spans="1:6" outlineLevel="1" collapsed="1">
       <c r="A119" s="13" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="B119" s="55"/>
       <c r="C119" s="13" t="s">
         <v>9</v>
       </c>
       <c r="D119" s="13" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E119" s="13" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="F119" s="13"/>
     </row>
     <row r="120" spans="1:6" outlineLevel="1">
       <c r="A120" s="21" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="B120" s="57"/>
       <c r="C120" s="21" t="s">
         <v>9</v>
       </c>
       <c r="D120" s="21" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E120" s="21" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="F120" s="21"/>
     </row>
     <row r="121" spans="1:6" outlineLevel="1">
       <c r="A121" s="13" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="B121" s="39"/>
       <c r="C121" s="13" t="s">
         <v>9</v>
       </c>
       <c r="D121" s="13" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E121" s="13" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="F121" s="13"/>
     </row>
     <row r="122" spans="1:6" outlineLevel="1" collapsed="1">
       <c r="A122" s="21" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="B122" s="57"/>
       <c r="C122" s="21" t="s">
         <v>9</v>
       </c>
       <c r="D122" s="21" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E122" s="21" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="F122" s="21"/>
     </row>
     <row r="123" spans="1:6" outlineLevel="1">
       <c r="A123" s="23" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="B123" s="61"/>
       <c r="C123" s="23" t="s">
         <v>9</v>
       </c>
       <c r="D123" s="23" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E123" s="23" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="F123" s="23"/>
     </row>
     <row r="124" spans="1:6" outlineLevel="1">
       <c r="A124" s="21" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="B124" s="57"/>
       <c r="C124" s="21" t="s">
         <v>9</v>
       </c>
       <c r="D124" s="21" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E124" s="21" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="F124" s="21"/>
     </row>
     <row r="125" spans="1:6" outlineLevel="1">
       <c r="A125" s="23" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="B125" s="61"/>
       <c r="C125" s="23" t="s">
         <v>9</v>
       </c>
       <c r="D125" s="23" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E125" s="23" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="F125" s="23"/>
     </row>
     <row r="126" spans="1:6" outlineLevel="1">
       <c r="A126" s="21" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="B126" s="57"/>
       <c r="C126" s="21" t="s">
         <v>9</v>
       </c>
       <c r="D126" s="21" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E126" s="21" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="F126" s="21"/>
     </row>
     <row r="127" spans="1:6" ht="14.45" customHeight="1">
       <c r="A127" s="36" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="B127" s="62"/>
       <c r="C127" s="25"/>
@@ -4374,7 +4373,7 @@
     </row>
     <row r="128" spans="1:6" outlineLevel="1">
       <c r="A128" s="14" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="B128" s="40"/>
       <c r="C128" s="14" t="s">
@@ -4384,118 +4383,114 @@
         <v>10</v>
       </c>
       <c r="E128" s="14" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="F128" s="14"/>
     </row>
     <row r="129" spans="1:8" outlineLevel="1">
       <c r="A129" s="13" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="B129" s="39"/>
       <c r="C129" s="13" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D129" s="13" t="s">
         <v>10</v>
       </c>
       <c r="E129" s="13" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="F129" s="13"/>
     </row>
     <row r="130" spans="1:8">
       <c r="A130" s="37" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="B130" s="63"/>
       <c r="C130" s="26"/>
       <c r="D130" s="26"/>
-      <c r="E130" s="26" t="s">
-        <v>11</v>
-      </c>
+      <c r="E130" s="26"/>
       <c r="F130" s="26"/>
     </row>
     <row r="131" spans="1:8" outlineLevel="1">
       <c r="A131" s="14" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="B131" s="40"/>
       <c r="C131" s="14" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D131" s="14" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E131" s="14" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="F131" s="14"/>
     </row>
     <row r="132" spans="1:8" outlineLevel="1">
       <c r="A132" s="13" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="B132" s="39"/>
       <c r="C132" s="13" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D132" s="13" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E132" s="13" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="F132" s="23"/>
       <c r="H132" s="12"/>
     </row>
     <row r="133" spans="1:8">
       <c r="A133" s="37" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="B133" s="63"/>
       <c r="C133" s="26"/>
       <c r="D133" s="26"/>
-      <c r="E133" s="26" t="s">
-        <v>11</v>
-      </c>
+      <c r="E133" s="26"/>
       <c r="F133" s="26"/>
     </row>
     <row r="134" spans="1:8" outlineLevel="1">
       <c r="A134" s="13" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="B134" s="39"/>
       <c r="C134" s="13" t="s">
         <v>9</v>
       </c>
       <c r="D134" s="13" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E134" s="13" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="F134" s="23"/>
     </row>
     <row r="135" spans="1:8" outlineLevel="1">
       <c r="A135" s="14" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="B135" s="40"/>
       <c r="C135" s="14" t="s">
         <v>9</v>
       </c>
       <c r="D135" s="14" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E135" s="14" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="F135" s="14"/>
     </row>
     <row r="136" spans="1:8">
       <c r="A136" s="36" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="B136" s="62"/>
       <c r="C136" s="25"/>
@@ -4505,7 +4500,7 @@
     </row>
     <row r="137" spans="1:8" outlineLevel="1">
       <c r="A137" s="14" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="B137" s="40"/>
       <c r="C137" s="14" t="s">
@@ -4515,13 +4510,13 @@
         <v>10</v>
       </c>
       <c r="E137" s="14" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="F137" s="14"/>
     </row>
     <row r="138" spans="1:8" outlineLevel="1">
       <c r="A138" s="13" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="B138" s="39"/>
       <c r="C138" s="13" t="s">
@@ -4531,13 +4526,13 @@
         <v>10</v>
       </c>
       <c r="E138" s="13" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="F138" s="13"/>
     </row>
     <row r="139" spans="1:8" outlineLevel="1">
       <c r="A139" s="14" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="B139" s="40"/>
       <c r="C139" s="14" t="s">
@@ -4547,13 +4542,13 @@
         <v>10</v>
       </c>
       <c r="E139" s="14" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="F139" s="14"/>
     </row>
     <row r="140" spans="1:8" outlineLevel="1">
       <c r="A140" s="13" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="B140" s="39"/>
       <c r="C140" s="13" t="s">
@@ -4563,157 +4558,157 @@
         <v>10</v>
       </c>
       <c r="E140" s="13" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="F140" s="13"/>
     </row>
     <row r="141" spans="1:8" outlineLevel="1">
       <c r="A141" s="14" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="B141" s="40"/>
       <c r="C141" s="14" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="D141" s="14" t="s">
         <v>10</v>
       </c>
       <c r="E141" s="14" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="F141" s="14"/>
     </row>
     <row r="142" spans="1:8" outlineLevel="1">
       <c r="A142" s="13" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="B142" s="39"/>
       <c r="C142" s="13" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="D142" s="13" t="s">
         <v>10</v>
       </c>
       <c r="E142" s="13" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="F142" s="13"/>
     </row>
     <row r="143" spans="1:8" outlineLevel="1">
       <c r="A143" s="14" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="B143" s="40"/>
       <c r="C143" s="14" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="D143" s="14" t="s">
         <v>10</v>
       </c>
       <c r="E143" s="27" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="F143" s="14"/>
     </row>
     <row r="144" spans="1:8" outlineLevel="1">
       <c r="A144" s="13" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="B144" s="39"/>
       <c r="C144" s="13" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="D144" s="13" t="s">
         <v>10</v>
       </c>
       <c r="E144" s="13" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="F144" s="13"/>
     </row>
     <row r="145" spans="1:6" outlineLevel="1">
       <c r="A145" s="14" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="B145" s="40"/>
       <c r="C145" s="14" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="D145" s="14" t="s">
         <v>10</v>
       </c>
       <c r="E145" s="14" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="F145" s="14"/>
     </row>
     <row r="146" spans="1:6" outlineLevel="1">
       <c r="A146" s="13" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="B146" s="39"/>
       <c r="C146" s="13" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="D146" s="13" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E146" s="13" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="F146" s="13"/>
     </row>
     <row r="147" spans="1:6" outlineLevel="1">
       <c r="A147" s="14" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="B147" s="40"/>
       <c r="C147" s="14" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="D147" s="14" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E147" s="14" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="F147" s="14"/>
     </row>
     <row r="148" spans="1:6" outlineLevel="1">
       <c r="A148" s="13" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="B148" s="39"/>
       <c r="C148" s="13" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="D148" s="13" t="s">
         <v>10</v>
       </c>
       <c r="E148" s="13" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="F148" s="13"/>
     </row>
     <row r="149" spans="1:6" outlineLevel="1">
       <c r="A149" s="14" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="B149" s="40"/>
       <c r="C149" s="14" t="s">
         <v>9</v>
       </c>
       <c r="D149" s="14" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E149" s="14" t="s">
-        <v>5</v>
+        <v>411</v>
       </c>
       <c r="F149" s="14"/>
     </row>
     <row r="150" spans="1:6">
       <c r="A150" s="37" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="B150" s="64"/>
       <c r="C150" s="26"/>
@@ -4723,33 +4718,33 @@
     </row>
     <row r="151" spans="1:6" outlineLevel="1">
       <c r="A151" s="13" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="B151" s="39"/>
       <c r="C151" s="13" t="s">
         <v>9</v>
       </c>
       <c r="D151" s="13" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E151" s="13" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="F151" s="13"/>
     </row>
     <row r="152" spans="1:6" outlineLevel="1">
       <c r="A152" s="14" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="B152" s="40"/>
       <c r="C152" s="14" t="s">
         <v>9</v>
       </c>
       <c r="D152" s="14" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E152" s="14" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="F152" s="14"/>
     </row>
@@ -4808,11 +4803,11 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D34">
-    <cfRule type="expression" dxfId="24" priority="22">
+    <cfRule type="expression" dxfId="24" priority="23">
+      <formula>$B29="Hide"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="23" priority="22">
       <formula>#REF!="Hide"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="23" priority="23">
-      <formula>$B29="Hide"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D38">
@@ -4871,11 +4866,11 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D80">
-    <cfRule type="expression" dxfId="11" priority="11">
+    <cfRule type="expression" dxfId="11" priority="12">
+      <formula>$B78="Hide"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="10" priority="11">
       <formula>$B76="Hide"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="10" priority="12">
-      <formula>$B78="Hide"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D81">
@@ -4939,66 +4934,66 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="6" t="s">
+        <v>264</v>
+      </c>
+      <c r="B1" s="6" t="s">
         <v>265</v>
-      </c>
-      <c r="B1" s="6" t="s">
-        <v>266</v>
       </c>
     </row>
     <row r="2" spans="1:2">
       <c r="A2" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
     </row>
     <row r="3" spans="1:2">
       <c r="A3" t="s">
+        <v>267</v>
+      </c>
+      <c r="B3" s="1" t="s">
         <v>268</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>269</v>
       </c>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" t="s">
+        <v>269</v>
+      </c>
+      <c r="B4" s="1" t="s">
         <v>270</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>271</v>
       </c>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" t="s">
+        <v>271</v>
+      </c>
+      <c r="B5" s="1" t="s">
         <v>272</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>273</v>
       </c>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" t="s">
+        <v>274</v>
+      </c>
+      <c r="B7" s="1" t="s">
         <v>275</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>276</v>
       </c>
     </row>
     <row r="8" spans="1:2">
       <c r="A8" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
     </row>
   </sheetData>
@@ -5025,145 +5020,145 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="11" t="s">
+        <v>264</v>
+      </c>
+      <c r="B1" s="11" t="s">
         <v>265</v>
-      </c>
-      <c r="B1" s="11" t="s">
-        <v>266</v>
       </c>
     </row>
     <row r="2" spans="1:2">
       <c r="A2" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="3" spans="1:2">
       <c r="A3" t="s">
+        <v>278</v>
+      </c>
+      <c r="B3" t="s">
         <v>279</v>
-      </c>
-      <c r="B3" t="s">
-        <v>280</v>
       </c>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" t="s">
+        <v>281</v>
+      </c>
+      <c r="B6" t="s">
         <v>282</v>
-      </c>
-      <c r="B6" t="s">
-        <v>283</v>
       </c>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" t="s">
+        <v>283</v>
+      </c>
+      <c r="B7" t="s">
         <v>284</v>
-      </c>
-      <c r="B7" t="s">
-        <v>285</v>
       </c>
     </row>
     <row r="8" spans="1:2">
       <c r="A8" t="s">
+        <v>285</v>
+      </c>
+      <c r="B8" t="s">
         <v>286</v>
-      </c>
-      <c r="B8" t="s">
-        <v>287</v>
       </c>
     </row>
     <row r="9" spans="1:2">
       <c r="A9" t="s">
+        <v>287</v>
+      </c>
+      <c r="B9" t="s">
         <v>288</v>
-      </c>
-      <c r="B9" t="s">
-        <v>289</v>
       </c>
     </row>
     <row r="10" spans="1:2">
       <c r="A10" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="B10" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="11" spans="1:2">
       <c r="A11" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="B11" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
     </row>
     <row r="12" spans="1:2">
       <c r="A12" t="s">
+        <v>290</v>
+      </c>
+      <c r="B12" t="s">
         <v>291</v>
-      </c>
-      <c r="B12" t="s">
-        <v>292</v>
       </c>
     </row>
     <row r="13" spans="1:2">
       <c r="A13" t="s">
+        <v>292</v>
+      </c>
+      <c r="B13" t="s">
         <v>293</v>
-      </c>
-      <c r="B13" t="s">
-        <v>294</v>
       </c>
     </row>
     <row r="14" spans="1:2">
       <c r="A14" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="B14" s="7"/>
     </row>
     <row r="15" spans="1:2">
       <c r="A15" s="2" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="B15" s="8"/>
     </row>
     <row r="16" spans="1:2">
       <c r="A16" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
     </row>
     <row r="17" spans="1:2">
       <c r="A17" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
     </row>
     <row r="18" spans="1:2">
       <c r="A18" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
     </row>
     <row r="19" spans="1:2">
       <c r="A19" t="s">
+        <v>299</v>
+      </c>
+      <c r="B19" t="s">
         <v>300</v>
-      </c>
-      <c r="B19" t="s">
-        <v>301</v>
       </c>
     </row>
     <row r="20" spans="1:2">
       <c r="A20" t="s">
+        <v>302</v>
+      </c>
+      <c r="B20" t="s">
         <v>303</v>
-      </c>
-      <c r="B20" t="s">
-        <v>304</v>
       </c>
     </row>
     <row r="21" spans="1:2">
       <c r="A21" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
     </row>
   </sheetData>
@@ -5189,206 +5184,206 @@
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" s="6" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="B1" s="6" t="s">
+        <v>326</v>
+      </c>
+      <c r="C1" s="6" t="s">
         <v>327</v>
-      </c>
-      <c r="C1" s="6" t="s">
-        <v>328</v>
       </c>
     </row>
     <row r="2" spans="1:3">
       <c r="A2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C2" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
     </row>
     <row r="3" spans="1:3">
       <c r="A3" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="4" spans="1:3">
       <c r="A4" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="C4" s="10" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
     </row>
     <row r="5" spans="1:3">
       <c r="A5" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="6" spans="1:3">
       <c r="A6" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="7" spans="1:3">
       <c r="A7" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="8" spans="1:3">
       <c r="A8" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="9" spans="1:3">
       <c r="A9" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
     </row>
     <row r="10" spans="1:3">
       <c r="A10" s="5" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
     </row>
     <row r="11" spans="1:3">
       <c r="A11" s="5" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
     </row>
     <row r="12" spans="1:3">
       <c r="A12" s="5" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
     </row>
     <row r="13" spans="1:3">
       <c r="A13" s="5" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
     </row>
     <row r="14" spans="1:3">
       <c r="A14" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
     </row>
     <row r="15" spans="1:3">
       <c r="A15" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
     </row>
     <row r="16" spans="1:3">
       <c r="A16" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B16" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
     </row>
     <row r="17" spans="1:2">
       <c r="A17" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="B17" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
     </row>
     <row r="18" spans="1:2">
       <c r="A18" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="B18" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
     </row>
     <row r="19" spans="1:2">
       <c r="A19" t="s">
+        <v>390</v>
+      </c>
+      <c r="B19" t="s">
         <v>391</v>
-      </c>
-      <c r="B19" t="s">
-        <v>392</v>
       </c>
     </row>
     <row r="20" spans="1:2">
       <c r="A20" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B20" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
     </row>
     <row r="21" spans="1:2">
       <c r="A21" t="s">
+        <v>336</v>
+      </c>
+      <c r="B21" s="10" t="s">
         <v>337</v>
-      </c>
-      <c r="B21" s="10" t="s">
-        <v>338</v>
       </c>
     </row>
     <row r="22" spans="1:2">
       <c r="A22" t="s">
+        <v>338</v>
+      </c>
+      <c r="B22" t="s">
         <v>339</v>
-      </c>
-      <c r="B22" t="s">
-        <v>340</v>
       </c>
     </row>
     <row r="23" spans="1:2">
       <c r="A23" t="s">
+        <v>340</v>
+      </c>
+      <c r="B23" t="s">
         <v>341</v>
-      </c>
-      <c r="B23" t="s">
-        <v>342</v>
       </c>
     </row>
     <row r="24" spans="1:2">
       <c r="A24" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
     <row r="25" spans="1:2">
       <c r="A25" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
     </row>
     <row r="26" spans="1:2">
       <c r="A26" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="27" spans="1:2">
       <c r="A27" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
     </row>
     <row r="28" spans="1:2">
       <c r="A28" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="29" spans="1:2">
       <c r="A29" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="30" spans="1:2">
       <c r="A30" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
     </row>
     <row r="31" spans="1:2">
       <c r="A31" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
     </row>
     <row r="32" spans="1:2">
       <c r="A32" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
     </row>
     <row r="33" spans="1:1">
       <c r="A33" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
     </row>
   </sheetData>
@@ -5411,154 +5406,154 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="6" t="s">
+        <v>264</v>
+      </c>
+      <c r="B1" s="6" t="s">
         <v>265</v>
-      </c>
-      <c r="B1" s="6" t="s">
-        <v>266</v>
       </c>
     </row>
     <row r="2" spans="1:2">
       <c r="A2" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="B2" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
     </row>
     <row r="3" spans="1:2">
       <c r="A3" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B3" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B4" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" t="s">
+        <v>307</v>
+      </c>
+      <c r="B5" s="3" t="s">
         <v>308</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>309</v>
       </c>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" t="s">
+        <v>309</v>
+      </c>
+      <c r="B6" s="3" t="s">
         <v>310</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>311</v>
       </c>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B7" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
     </row>
     <row r="8" spans="1:2">
       <c r="A8" t="s">
+        <v>312</v>
+      </c>
+      <c r="B8" t="s">
         <v>313</v>
-      </c>
-      <c r="B8" t="s">
-        <v>314</v>
       </c>
     </row>
     <row r="9" spans="1:2">
       <c r="A9" t="s">
+        <v>314</v>
+      </c>
+      <c r="B9" t="s">
         <v>315</v>
-      </c>
-      <c r="B9" t="s">
-        <v>316</v>
       </c>
     </row>
     <row r="10" spans="1:2">
       <c r="A10" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B10" s="9" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
     </row>
     <row r="11" spans="1:2">
       <c r="A11" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B11" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
     </row>
     <row r="12" spans="1:2">
       <c r="A12" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B12" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
     </row>
     <row r="13" spans="1:2">
       <c r="A13" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B13" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
     </row>
     <row r="14" spans="1:2">
       <c r="A14" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="B14" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
     </row>
     <row r="15" spans="1:2">
       <c r="A15" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B15" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
     </row>
     <row r="16" spans="1:2">
       <c r="A16" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="B16" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
     </row>
     <row r="17" spans="1:2">
       <c r="A17" s="2" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
     </row>
     <row r="18" spans="1:2">
       <c r="A18" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
     </row>
     <row r="19" spans="1:2">
       <c r="A19" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B19" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
     </row>
   </sheetData>
@@ -5567,68 +5562,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <FolderType xmlns="35345429-01ed-4d83-85b9-6cc21878d784" xsi:nil="true"/>
-    <CultureName xmlns="35345429-01ed-4d83-85b9-6cc21878d784" xsi:nil="true"/>
-    <Leaders xmlns="35345429-01ed-4d83-85b9-6cc21878d784">
-      <UserInfo>
-        <DisplayName/>
-        <AccountId xsi:nil="true"/>
-        <AccountType/>
-      </UserInfo>
-    </Leaders>
-    <IsNotebookLocked xmlns="35345429-01ed-4d83-85b9-6cc21878d784" xsi:nil="true"/>
-    <Invited_Members xmlns="35345429-01ed-4d83-85b9-6cc21878d784" xsi:nil="true"/>
-    <Math_Settings xmlns="35345429-01ed-4d83-85b9-6cc21878d784" xsi:nil="true"/>
-    <Self_Registration_Enabled xmlns="35345429-01ed-4d83-85b9-6cc21878d784" xsi:nil="true"/>
-    <Has_Leaders_Only_SectionGroup xmlns="35345429-01ed-4d83-85b9-6cc21878d784" xsi:nil="true"/>
-    <Member_Groups xmlns="35345429-01ed-4d83-85b9-6cc21878d784">
-      <UserInfo>
-        <DisplayName/>
-        <AccountId xsi:nil="true"/>
-        <AccountType/>
-      </UserInfo>
-    </Member_Groups>
-    <Distribution_Groups xmlns="35345429-01ed-4d83-85b9-6cc21878d784" xsi:nil="true"/>
-    <AppVersion xmlns="35345429-01ed-4d83-85b9-6cc21878d784" xsi:nil="true"/>
-    <DefaultSectionNames xmlns="35345429-01ed-4d83-85b9-6cc21878d784" xsi:nil="true"/>
-    <Templates xmlns="35345429-01ed-4d83-85b9-6cc21878d784" xsi:nil="true"/>
-    <NotebookType xmlns="35345429-01ed-4d83-85b9-6cc21878d784" xsi:nil="true"/>
-    <TeamsChannelId xmlns="35345429-01ed-4d83-85b9-6cc21878d784" xsi:nil="true"/>
-    <Invited_Leaders xmlns="35345429-01ed-4d83-85b9-6cc21878d784" xsi:nil="true"/>
-    <Is_Collaboration_Space_Locked xmlns="35345429-01ed-4d83-85b9-6cc21878d784" xsi:nil="true"/>
-    <Teams_Channel_Section_Location xmlns="35345429-01ed-4d83-85b9-6cc21878d784" xsi:nil="true"/>
-    <Members xmlns="35345429-01ed-4d83-85b9-6cc21878d784">
-      <UserInfo>
-        <DisplayName/>
-        <AccountId xsi:nil="true"/>
-        <AccountType/>
-      </UserInfo>
-    </Members>
-    <Owner xmlns="35345429-01ed-4d83-85b9-6cc21878d784">
-      <UserInfo>
-        <DisplayName/>
-        <AccountId xsi:nil="true"/>
-        <AccountType/>
-      </UserInfo>
-    </Owner>
-    <LMS_Mappings xmlns="35345429-01ed-4d83-85b9-6cc21878d784" xsi:nil="true"/>
-    <_activity xmlns="35345429-01ed-4d83-85b9-6cc21878d784" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Dokument" ma:contentTypeID="0x010100F5BD758A7F2BF742ADB9291A93682A9E" ma:contentTypeVersion="31" ma:contentTypeDescription="Ein neues Dokument erstellen." ma:contentTypeScope="" ma:versionID="0517f02299b6dbd064809d9c3f869e8a">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="35345429-01ed-4d83-85b9-6cc21878d784" xmlns:ns4="53f86fb7-11c0-476e-bf8b-57768422e991" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="a7ff6e993c77c55b2c02ebba747ae01b" ns3:_="" ns4:_="">
     <xsd:import namespace="35345429-01ed-4d83-85b9-6cc21878d784"/>
@@ -6025,25 +5958,69 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E85C156E-EE0C-426A-92B3-CAF84DB17690}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B2D89A20-922B-4399-8A99-02ABCC3D1E33}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="35345429-01ed-4d83-85b9-6cc21878d784"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <FolderType xmlns="35345429-01ed-4d83-85b9-6cc21878d784" xsi:nil="true"/>
+    <CultureName xmlns="35345429-01ed-4d83-85b9-6cc21878d784" xsi:nil="true"/>
+    <Leaders xmlns="35345429-01ed-4d83-85b9-6cc21878d784">
+      <UserInfo>
+        <DisplayName/>
+        <AccountId xsi:nil="true"/>
+        <AccountType/>
+      </UserInfo>
+    </Leaders>
+    <IsNotebookLocked xmlns="35345429-01ed-4d83-85b9-6cc21878d784" xsi:nil="true"/>
+    <Invited_Members xmlns="35345429-01ed-4d83-85b9-6cc21878d784" xsi:nil="true"/>
+    <Math_Settings xmlns="35345429-01ed-4d83-85b9-6cc21878d784" xsi:nil="true"/>
+    <Self_Registration_Enabled xmlns="35345429-01ed-4d83-85b9-6cc21878d784" xsi:nil="true"/>
+    <Has_Leaders_Only_SectionGroup xmlns="35345429-01ed-4d83-85b9-6cc21878d784" xsi:nil="true"/>
+    <Member_Groups xmlns="35345429-01ed-4d83-85b9-6cc21878d784">
+      <UserInfo>
+        <DisplayName/>
+        <AccountId xsi:nil="true"/>
+        <AccountType/>
+      </UserInfo>
+    </Member_Groups>
+    <Distribution_Groups xmlns="35345429-01ed-4d83-85b9-6cc21878d784" xsi:nil="true"/>
+    <AppVersion xmlns="35345429-01ed-4d83-85b9-6cc21878d784" xsi:nil="true"/>
+    <DefaultSectionNames xmlns="35345429-01ed-4d83-85b9-6cc21878d784" xsi:nil="true"/>
+    <Templates xmlns="35345429-01ed-4d83-85b9-6cc21878d784" xsi:nil="true"/>
+    <NotebookType xmlns="35345429-01ed-4d83-85b9-6cc21878d784" xsi:nil="true"/>
+    <TeamsChannelId xmlns="35345429-01ed-4d83-85b9-6cc21878d784" xsi:nil="true"/>
+    <Invited_Leaders xmlns="35345429-01ed-4d83-85b9-6cc21878d784" xsi:nil="true"/>
+    <Is_Collaboration_Space_Locked xmlns="35345429-01ed-4d83-85b9-6cc21878d784" xsi:nil="true"/>
+    <Teams_Channel_Section_Location xmlns="35345429-01ed-4d83-85b9-6cc21878d784" xsi:nil="true"/>
+    <Members xmlns="35345429-01ed-4d83-85b9-6cc21878d784">
+      <UserInfo>
+        <DisplayName/>
+        <AccountId xsi:nil="true"/>
+        <AccountType/>
+      </UserInfo>
+    </Members>
+    <Owner xmlns="35345429-01ed-4d83-85b9-6cc21878d784">
+      <UserInfo>
+        <DisplayName/>
+        <AccountId xsi:nil="true"/>
+        <AccountType/>
+      </UserInfo>
+    </Owner>
+    <LMS_Mappings xmlns="35345429-01ed-4d83-85b9-6cc21878d784" xsi:nil="true"/>
+    <_activity xmlns="35345429-01ed-4d83-85b9-6cc21878d784" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0D716C96-A80E-4732-A5D3-9C77E88EE8CA}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -6060,4 +6037,22 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E85C156E-EE0C-426A-92B3-CAF84DB17690}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B2D89A20-922B-4399-8A99-02ABCC3D1E33}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="35345429-01ed-4d83-85b9-6cc21878d784"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Update schema: `Cell label` -> `Cell name`
</commit_message>
<xml_diff>
--- a/Excel for reference/BattINFO_converter_standard_Excel_version_1.1.17_empty.xlsx
+++ b/Excel for reference/BattINFO_converter_standard_Excel_version_1.1.17_empty.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\battinfoconverter\Excel for reference\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C5113F5C-C60B-4434-9E80-5594AAD21078}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9386ED2-9E6C-41A3-A72C-520A1FF6F5ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="19200" yWindow="3945" windowWidth="24060" windowHeight="16140" xr2:uid="{1A6D523C-FE67-4F3F-AA9B-E9FEE83DA8F2}"/>
+    <workbookView xWindow="4575" yWindow="2280" windowWidth="23985" windowHeight="16935" xr2:uid="{1A6D523C-FE67-4F3F-AA9B-E9FEE83DA8F2}"/>
   </bookViews>
   <sheets>
     <sheet name="@Schema" sheetId="2" r:id="rId1"/>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="709" uniqueCount="415">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="703" uniqueCount="411">
   <si>
     <t>Metadata</t>
   </si>
@@ -1237,33 +1237,12 @@
     <t>REQUIRED, CANNOT BE CHANGED</t>
   </si>
   <si>
-    <t>empa__ccid_123456</t>
-  </si>
-  <si>
-    <t>Cell label</t>
-  </si>
-  <si>
-    <t>rdfs:label</t>
-  </si>
-  <si>
-    <t>Human-friendly name or label for cell</t>
-  </si>
-  <si>
-    <t>Battery2030+/PREMISE</t>
-  </si>
-  <si>
-    <t>manually</t>
-  </si>
-  <si>
     <t>Name of this CoinCell Schema, do not change</t>
   </si>
   <si>
     <t>Version of this CoinCell Schema, do not change</t>
   </si>
   <si>
-    <t>240616_bco_gr-NMC_01</t>
-  </si>
-  <si>
     <t>type|</t>
   </si>
   <si>
@@ -1289,6 +1268,15 @@
   </si>
   <si>
     <t>REQUIRED, CANNOT BE CHANGED, value should be in @classes with ID</t>
+  </si>
+  <si>
+    <t>Cell name</t>
+  </si>
+  <si>
+    <t>schema:name</t>
+  </si>
+  <si>
+    <t>Human-friendly name for the cell</t>
   </si>
 </sst>
 </file>
@@ -2421,7 +2409,7 @@
         <v>10</v>
       </c>
       <c r="E3" s="13" t="s">
-        <v>406</v>
+        <v>399</v>
       </c>
       <c r="F3" s="13" t="s">
         <v>396</v>
@@ -2431,9 +2419,7 @@
       <c r="A4" s="14" t="s">
         <v>11</v>
       </c>
-      <c r="B4" s="40" t="s">
-        <v>397</v>
-      </c>
+      <c r="B4" s="40"/>
       <c r="C4" s="14" t="s">
         <v>9</v>
       </c>
@@ -2441,19 +2427,17 @@
         <v>10</v>
       </c>
       <c r="E4" s="14" t="s">
-        <v>407</v>
+        <v>400</v>
       </c>
       <c r="F4" s="14" t="s">
-        <v>412</v>
+        <v>405</v>
       </c>
     </row>
     <row r="5" spans="1:6" outlineLevel="1">
       <c r="A5" s="13" t="s">
-        <v>398</v>
-      </c>
-      <c r="B5" s="39" t="s">
-        <v>405</v>
-      </c>
+        <v>408</v>
+      </c>
+      <c r="B5" s="39"/>
       <c r="C5" s="13" t="s">
         <v>9</v>
       </c>
@@ -2461,19 +2445,17 @@
         <v>18</v>
       </c>
       <c r="E5" s="13" t="s">
-        <v>399</v>
+        <v>409</v>
       </c>
       <c r="F5" s="13" t="s">
-        <v>400</v>
+        <v>410</v>
       </c>
     </row>
     <row r="6" spans="1:6" outlineLevel="1">
       <c r="A6" s="14" t="s">
         <v>12</v>
       </c>
-      <c r="B6" s="66">
-        <v>45459</v>
-      </c>
+      <c r="B6" s="66"/>
       <c r="C6" s="14" t="s">
         <v>9</v>
       </c>
@@ -2481,19 +2463,17 @@
         <v>10</v>
       </c>
       <c r="E6" s="14" t="s">
-        <v>408</v>
+        <v>401</v>
       </c>
       <c r="F6" s="14" t="s">
-        <v>413</v>
+        <v>406</v>
       </c>
     </row>
     <row r="7" spans="1:6" outlineLevel="1">
       <c r="A7" s="13" t="s">
         <v>13</v>
       </c>
-      <c r="B7" s="39" t="s">
-        <v>14</v>
-      </c>
+      <c r="B7" s="39"/>
       <c r="C7" s="13" t="s">
         <v>9</v>
       </c>
@@ -2501,19 +2481,17 @@
         <v>10</v>
       </c>
       <c r="E7" s="13" t="s">
-        <v>409</v>
+        <v>402</v>
       </c>
       <c r="F7" s="13" t="s">
-        <v>414</v>
+        <v>407</v>
       </c>
     </row>
     <row r="8" spans="1:6" outlineLevel="1">
       <c r="A8" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="B8" s="40" t="s">
-        <v>16</v>
-      </c>
+      <c r="B8" s="40"/>
       <c r="C8" s="14" t="s">
         <v>9</v>
       </c>
@@ -2521,19 +2499,17 @@
         <v>10</v>
       </c>
       <c r="E8" s="14" t="s">
-        <v>410</v>
+        <v>403</v>
       </c>
       <c r="F8" s="14" t="s">
-        <v>414</v>
+        <v>407</v>
       </c>
     </row>
     <row r="9" spans="1:6" outlineLevel="1">
       <c r="A9" s="13" t="s">
         <v>17</v>
       </c>
-      <c r="B9" s="39" t="s">
-        <v>401</v>
-      </c>
+      <c r="B9" s="39"/>
       <c r="C9" s="13" t="s">
         <v>9</v>
       </c>
@@ -2541,7 +2517,7 @@
         <v>18</v>
       </c>
       <c r="E9" s="13" t="s">
-        <v>411</v>
+        <v>404</v>
       </c>
       <c r="F9" s="13"/>
     </row>
@@ -2549,9 +2525,7 @@
       <c r="A10" s="14" t="s">
         <v>19</v>
       </c>
-      <c r="B10" s="40" t="s">
-        <v>402</v>
-      </c>
+      <c r="B10" s="40"/>
       <c r="C10" s="14" t="s">
         <v>9</v>
       </c>
@@ -2559,7 +2533,7 @@
         <v>18</v>
       </c>
       <c r="E10" s="14" t="s">
-        <v>411</v>
+        <v>404</v>
       </c>
       <c r="F10" s="14"/>
     </row>
@@ -2577,10 +2551,10 @@
         <v>10</v>
       </c>
       <c r="E11" s="13" t="s">
-        <v>411</v>
+        <v>404</v>
       </c>
       <c r="F11" s="13" t="s">
-        <v>403</v>
+        <v>397</v>
       </c>
     </row>
     <row r="12" spans="1:6" outlineLevel="1">
@@ -2597,10 +2571,10 @@
         <v>10</v>
       </c>
       <c r="E12" s="14" t="s">
-        <v>411</v>
+        <v>404</v>
       </c>
       <c r="F12" s="14" t="s">
-        <v>404</v>
+        <v>398</v>
       </c>
     </row>
     <row r="13" spans="1:6">
@@ -4702,7 +4676,7 @@
         <v>50</v>
       </c>
       <c r="E149" s="14" t="s">
-        <v>411</v>
+        <v>404</v>
       </c>
       <c r="F149" s="14"/>
     </row>
@@ -5562,6 +5536,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Dokument" ma:contentTypeID="0x010100F5BD758A7F2BF742ADB9291A93682A9E" ma:contentTypeVersion="31" ma:contentTypeDescription="Ein neues Dokument erstellen." ma:contentTypeScope="" ma:versionID="0517f02299b6dbd064809d9c3f869e8a">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="35345429-01ed-4d83-85b9-6cc21878d784" xmlns:ns4="53f86fb7-11c0-476e-bf8b-57768422e991" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="a7ff6e993c77c55b2c02ebba747ae01b" ns3:_="" ns4:_="">
     <xsd:import namespace="35345429-01ed-4d83-85b9-6cc21878d784"/>
@@ -5958,15 +5941,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -6021,6 +5995,14 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E85C156E-EE0C-426A-92B3-CAF84DB17690}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0D716C96-A80E-4732-A5D3-9C77E88EE8CA}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -6039,14 +6021,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E85C156E-EE0C-426A-92B3-CAF84DB17690}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B2D89A20-922B-4399-8A99-02ABCC3D1E33}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
Remove hardcoded header (#64)
* Remove required hardcoded NotOntologize terms

Allows normal ontology link at root level

* Add hardcoded backwards compatibility tests

* Update schema, drop all NotOntologize, adds `Cell name`

* Clearer manufacturer/creator warning
</commit_message>
<xml_diff>
--- a/Excel for reference/BattINFO_converter_standard_Excel_version_1.1.17_empty.xlsx
+++ b/Excel for reference/BattINFO_converter_standard_Excel_version_1.1.17_empty.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\battinfoconverter\Excel for reference\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01AA420C-455B-4972-9AA5-ADD5D46552FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9386ED2-9E6C-41A3-A72C-520A1FF6F5ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="25695" yWindow="0" windowWidth="26010" windowHeight="20985" xr2:uid="{1A6D523C-FE67-4F3F-AA9B-E9FEE83DA8F2}"/>
+    <workbookView xWindow="4575" yWindow="2280" windowWidth="23985" windowHeight="16935" xr2:uid="{1A6D523C-FE67-4F3F-AA9B-E9FEE83DA8F2}"/>
   </bookViews>
   <sheets>
     <sheet name="@Schema" sheetId="2" r:id="rId1"/>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="719" uniqueCount="410">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="703" uniqueCount="411">
   <si>
     <t>Metadata</t>
   </si>
@@ -79,9 +79,6 @@
     <t>required</t>
   </si>
   <si>
-    <t>NotOntologize</t>
-  </si>
-  <si>
     <t>Cell ID</t>
   </si>
   <si>
@@ -1240,40 +1237,46 @@
     <t>REQUIRED, CANNOT BE CHANGED</t>
   </si>
   <si>
-    <t>empa__ccid_123456</t>
-  </si>
-  <si>
-    <t>REQUIRED, CANNOT BE CHANGED. Unique ID for cell.</t>
-  </si>
-  <si>
-    <t>Cell label</t>
-  </si>
-  <si>
-    <t>rdfs:label</t>
-  </si>
-  <si>
-    <t>Human-friendly name or label for cell</t>
-  </si>
-  <si>
-    <t>REQUIRED, CANNOT BE CHANGED. Value should be in @classes with ID</t>
-  </si>
-  <si>
-    <t>Battery2030+/PREMISE</t>
-  </si>
-  <si>
-    <t>manually</t>
-  </si>
-  <si>
     <t>Name of this CoinCell Schema, do not change</t>
   </si>
   <si>
     <t>Version of this CoinCell Schema, do not change</t>
   </si>
   <si>
-    <t>240616_bco_gr-NMC_01</t>
-  </si>
-  <si>
-    <t>REQUIRED, CANNOT BE CHANGED. Assembly date in ISO8601 format (YYYY-MM-DD).</t>
+    <t>type|</t>
+  </si>
+  <si>
+    <t>schema:productID</t>
+  </si>
+  <si>
+    <t>schema:dateCreated</t>
+  </si>
+  <si>
+    <t>schema:manufacturer</t>
+  </si>
+  <si>
+    <t>schema:creator</t>
+  </si>
+  <si>
+    <t>rdfs:comment</t>
+  </si>
+  <si>
+    <t>REQUIRED, CANNOT BE CHANGED, unique ID for cell</t>
+  </si>
+  <si>
+    <t>REQUIRED, CANNOT BE CHANGED, assembly date in ISO8601 format (YYYY-MM-DD)</t>
+  </si>
+  <si>
+    <t>REQUIRED, CANNOT BE CHANGED, value should be in @classes with ID</t>
+  </si>
+  <si>
+    <t>Cell name</t>
+  </si>
+  <si>
+    <t>schema:name</t>
+  </si>
+  <si>
+    <t>Human-friendly name for the cell</t>
   </si>
 </sst>
 </file>
@@ -1282,7 +1285,7 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
     <numFmt numFmtId="164" formatCode="0.0"/>
-    <numFmt numFmtId="166" formatCode="yyyy\-mm\-dd;@"/>
+    <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd;@"/>
   </numFmts>
   <fonts count="13">
     <font>
@@ -1658,7 +1661,7 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="4" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="4" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2406,19 +2409,17 @@
         <v>10</v>
       </c>
       <c r="E3" s="13" t="s">
-        <v>11</v>
+        <v>399</v>
       </c>
       <c r="F3" s="13" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="15" customHeight="1" outlineLevel="1">
       <c r="A4" s="14" t="s">
-        <v>12</v>
-      </c>
-      <c r="B4" s="40" t="s">
-        <v>398</v>
-      </c>
+        <v>11</v>
+      </c>
+      <c r="B4" s="40"/>
       <c r="C4" s="14" t="s">
         <v>9</v>
       </c>
@@ -2426,39 +2427,35 @@
         <v>10</v>
       </c>
       <c r="E4" s="14" t="s">
-        <v>11</v>
+        <v>400</v>
       </c>
       <c r="F4" s="14" t="s">
-        <v>399</v>
+        <v>405</v>
       </c>
     </row>
     <row r="5" spans="1:6" outlineLevel="1">
       <c r="A5" s="13" t="s">
-        <v>400</v>
-      </c>
-      <c r="B5" s="39" t="s">
         <v>408</v>
       </c>
+      <c r="B5" s="39"/>
       <c r="C5" s="13" t="s">
         <v>9</v>
       </c>
       <c r="D5" s="13" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E5" s="13" t="s">
-        <v>401</v>
+        <v>409</v>
       </c>
       <c r="F5" s="13" t="s">
-        <v>402</v>
+        <v>410</v>
       </c>
     </row>
     <row r="6" spans="1:6" outlineLevel="1">
       <c r="A6" s="14" t="s">
-        <v>13</v>
-      </c>
-      <c r="B6" s="66">
-        <v>45459</v>
-      </c>
+        <v>12</v>
+      </c>
+      <c r="B6" s="66"/>
       <c r="C6" s="14" t="s">
         <v>9</v>
       </c>
@@ -2466,19 +2463,17 @@
         <v>10</v>
       </c>
       <c r="E6" s="14" t="s">
-        <v>11</v>
+        <v>401</v>
       </c>
       <c r="F6" s="14" t="s">
-        <v>409</v>
+        <v>406</v>
       </c>
     </row>
     <row r="7" spans="1:6" outlineLevel="1">
       <c r="A7" s="13" t="s">
-        <v>14</v>
-      </c>
-      <c r="B7" s="39" t="s">
-        <v>15</v>
-      </c>
+        <v>13</v>
+      </c>
+      <c r="B7" s="39"/>
       <c r="C7" s="13" t="s">
         <v>9</v>
       </c>
@@ -2486,19 +2481,17 @@
         <v>10</v>
       </c>
       <c r="E7" s="13" t="s">
-        <v>11</v>
-      </c>
-      <c r="F7" s="14" t="s">
-        <v>403</v>
+        <v>402</v>
+      </c>
+      <c r="F7" s="13" t="s">
+        <v>407</v>
       </c>
     </row>
     <row r="8" spans="1:6" outlineLevel="1">
       <c r="A8" s="14" t="s">
-        <v>16</v>
-      </c>
-      <c r="B8" s="40" t="s">
-        <v>17</v>
-      </c>
+        <v>15</v>
+      </c>
+      <c r="B8" s="40"/>
       <c r="C8" s="14" t="s">
         <v>9</v>
       </c>
@@ -2506,54 +2499,50 @@
         <v>10</v>
       </c>
       <c r="E8" s="14" t="s">
-        <v>11</v>
+        <v>403</v>
       </c>
       <c r="F8" s="14" t="s">
-        <v>403</v>
+        <v>407</v>
       </c>
     </row>
     <row r="9" spans="1:6" outlineLevel="1">
       <c r="A9" s="13" t="s">
+        <v>17</v>
+      </c>
+      <c r="B9" s="39"/>
+      <c r="C9" s="13" t="s">
+        <v>9</v>
+      </c>
+      <c r="D9" s="13" t="s">
         <v>18</v>
       </c>
-      <c r="B9" s="39" t="s">
+      <c r="E9" s="13" t="s">
         <v>404</v>
-      </c>
-      <c r="C9" s="13" t="s">
-        <v>9</v>
-      </c>
-      <c r="D9" s="13" t="s">
-        <v>19</v>
-      </c>
-      <c r="E9" s="13" t="s">
-        <v>5</v>
       </c>
       <c r="F9" s="13"/>
     </row>
     <row r="10" spans="1:6" outlineLevel="1">
       <c r="A10" s="14" t="s">
-        <v>20</v>
-      </c>
-      <c r="B10" s="40" t="s">
-        <v>405</v>
-      </c>
+        <v>19</v>
+      </c>
+      <c r="B10" s="40"/>
       <c r="C10" s="14" t="s">
         <v>9</v>
       </c>
       <c r="D10" s="14" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E10" s="14" t="s">
-        <v>5</v>
+        <v>404</v>
       </c>
       <c r="F10" s="14"/>
     </row>
     <row r="11" spans="1:6" outlineLevel="1">
       <c r="A11" s="13" t="s">
+        <v>388</v>
+      </c>
+      <c r="B11" s="39" t="s">
         <v>389</v>
-      </c>
-      <c r="B11" s="39" t="s">
-        <v>390</v>
       </c>
       <c r="C11" s="13" t="s">
         <v>9</v>
@@ -2562,18 +2551,18 @@
         <v>10</v>
       </c>
       <c r="E11" s="13" t="s">
-        <v>5</v>
+        <v>404</v>
       </c>
       <c r="F11" s="13" t="s">
-        <v>406</v>
+        <v>397</v>
       </c>
     </row>
     <row r="12" spans="1:6" outlineLevel="1">
       <c r="A12" s="14" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="B12" s="40" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="C12" s="14" t="s">
         <v>9</v>
@@ -2582,15 +2571,15 @@
         <v>10</v>
       </c>
       <c r="E12" s="14" t="s">
-        <v>5</v>
+        <v>404</v>
       </c>
       <c r="F12" s="14" t="s">
-        <v>407</v>
+        <v>398</v>
       </c>
     </row>
     <row r="13" spans="1:6">
       <c r="A13" s="30" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B13" s="41"/>
       <c r="C13" s="15"/>
@@ -2600,7 +2589,7 @@
     </row>
     <row r="14" spans="1:6" outlineLevel="1">
       <c r="A14" s="13" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B14" s="39"/>
       <c r="C14" s="13" t="s">
@@ -2610,29 +2599,29 @@
         <v>10</v>
       </c>
       <c r="E14" s="13" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F14" s="13"/>
     </row>
     <row r="15" spans="1:6" outlineLevel="1">
       <c r="A15" s="16" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B15" s="42"/>
       <c r="C15" s="16" t="s">
+        <v>25</v>
+      </c>
+      <c r="D15" s="16" t="s">
+        <v>18</v>
+      </c>
+      <c r="E15" s="16" t="s">
         <v>26</v>
-      </c>
-      <c r="D15" s="16" t="s">
-        <v>19</v>
-      </c>
-      <c r="E15" s="16" t="s">
-        <v>27</v>
       </c>
       <c r="F15" s="16"/>
     </row>
     <row r="16" spans="1:6" outlineLevel="1">
       <c r="A16" s="13" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B16" s="39"/>
       <c r="C16" s="13" t="s">
@@ -2642,45 +2631,45 @@
         <v>10</v>
       </c>
       <c r="E16" s="13" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F16" s="13"/>
     </row>
     <row r="17" spans="1:6" outlineLevel="1">
       <c r="A17" s="16" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B17" s="42"/>
       <c r="C17" s="16" t="s">
         <v>9</v>
       </c>
       <c r="D17" s="16" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E17" s="16" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="F17" s="16"/>
     </row>
     <row r="18" spans="1:6" outlineLevel="1">
       <c r="A18" s="13" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B18" s="39"/>
       <c r="C18" s="13" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D18" s="13" t="s">
         <v>10</v>
       </c>
       <c r="E18" s="13" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="F18" s="13"/>
     </row>
     <row r="19" spans="1:6" outlineLevel="1">
       <c r="A19" s="16" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B19" s="42"/>
       <c r="C19" s="16" t="s">
@@ -2690,29 +2679,29 @@
         <v>10</v>
       </c>
       <c r="E19" s="16" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="F19" s="16"/>
     </row>
     <row r="20" spans="1:6" outlineLevel="1">
       <c r="A20" s="13" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B20" s="39"/>
       <c r="C20" s="13" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D20" s="13" t="s">
         <v>10</v>
       </c>
       <c r="E20" s="13" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="F20" s="13"/>
     </row>
     <row r="21" spans="1:6" ht="15.75" customHeight="1" outlineLevel="1">
       <c r="A21" s="16" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B21" s="42"/>
       <c r="C21" s="16" t="s">
@@ -2722,513 +2711,507 @@
         <v>10</v>
       </c>
       <c r="E21" s="16" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F21" s="16"/>
     </row>
     <row r="22" spans="1:6" outlineLevel="1">
       <c r="A22" s="13" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B22" s="39"/>
       <c r="C22" s="13" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D22" s="13" t="s">
         <v>10</v>
       </c>
       <c r="E22" s="13" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="F22" s="13"/>
     </row>
     <row r="23" spans="1:6" outlineLevel="1">
       <c r="A23" s="16" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B23" s="42"/>
       <c r="C23" s="16" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D23" s="16" t="s">
         <v>10</v>
       </c>
       <c r="E23" s="16" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="F23" s="16"/>
     </row>
     <row r="24" spans="1:6" outlineLevel="1">
       <c r="A24" s="13" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B24" s="39"/>
       <c r="C24" s="13" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D24" s="13" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E24" s="13" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="F24" s="13"/>
     </row>
     <row r="25" spans="1:6">
       <c r="A25" s="31" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B25" s="43"/>
       <c r="C25" s="15"/>
       <c r="D25" s="15"/>
-      <c r="E25" s="15" t="s">
-        <v>11</v>
-      </c>
+      <c r="E25" s="15"/>
       <c r="F25" s="15"/>
     </row>
     <row r="26" spans="1:6" outlineLevel="1">
       <c r="A26" s="13" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B26" s="39"/>
       <c r="C26" s="13" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D26" s="13" t="s">
+        <v>50</v>
+      </c>
+      <c r="E26" s="13" t="s">
         <v>51</v>
-      </c>
-      <c r="E26" s="13" t="s">
-        <v>52</v>
       </c>
       <c r="F26" s="13"/>
     </row>
     <row r="27" spans="1:6" outlineLevel="1">
       <c r="A27" s="16" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B27" s="44"/>
       <c r="C27" s="16" t="s">
+        <v>53</v>
+      </c>
+      <c r="D27" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="E27" s="16" t="s">
         <v>54</v>
-      </c>
-      <c r="D27" s="16" t="s">
-        <v>51</v>
-      </c>
-      <c r="E27" s="16" t="s">
-        <v>55</v>
       </c>
       <c r="F27" s="16"/>
     </row>
     <row r="28" spans="1:6" outlineLevel="1">
       <c r="A28" s="13" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B28" s="39"/>
       <c r="C28" s="13" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D28" s="13" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E28" s="13" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="F28" s="13"/>
     </row>
     <row r="29" spans="1:6">
       <c r="A29" s="31" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B29" s="43"/>
       <c r="C29" s="15"/>
       <c r="D29" s="15"/>
-      <c r="E29" s="15" t="s">
-        <v>11</v>
-      </c>
+      <c r="E29" s="15"/>
       <c r="F29" s="15"/>
     </row>
     <row r="30" spans="1:6" outlineLevel="1">
       <c r="A30" s="13" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B30" s="39"/>
       <c r="C30" s="13" t="s">
         <v>9</v>
       </c>
       <c r="D30" s="13" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E30" s="13" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="F30" s="13"/>
     </row>
     <row r="31" spans="1:6" outlineLevel="1">
       <c r="A31" s="16" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B31" s="42"/>
       <c r="C31" s="16" t="s">
         <v>9</v>
       </c>
       <c r="D31" s="16" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E31" s="16" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="F31" s="16"/>
     </row>
     <row r="32" spans="1:6" outlineLevel="1">
       <c r="A32" s="13" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B32" s="45"/>
       <c r="C32" s="13" t="s">
+        <v>64</v>
+      </c>
+      <c r="D32" s="13" t="s">
+        <v>50</v>
+      </c>
+      <c r="E32" s="13" t="s">
         <v>65</v>
-      </c>
-      <c r="D32" s="13" t="s">
-        <v>51</v>
-      </c>
-      <c r="E32" s="13" t="s">
-        <v>66</v>
       </c>
       <c r="F32" s="13"/>
     </row>
     <row r="33" spans="1:6" outlineLevel="1">
       <c r="A33" s="16" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B33" s="42"/>
       <c r="C33" s="16" t="s">
+        <v>67</v>
+      </c>
+      <c r="D33" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="E33" s="16" t="s">
         <v>68</v>
-      </c>
-      <c r="D33" s="16" t="s">
-        <v>51</v>
-      </c>
-      <c r="E33" s="16" t="s">
-        <v>69</v>
       </c>
       <c r="F33" s="16"/>
     </row>
     <row r="34" spans="1:6" outlineLevel="1">
       <c r="A34" s="13" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B34" s="39"/>
       <c r="C34" s="13" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D34" s="13" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E34" s="13" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="F34" s="13"/>
     </row>
     <row r="35" spans="1:6" outlineLevel="1">
       <c r="A35" s="16" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B35" s="42"/>
       <c r="C35" s="16" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D35" s="16" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E35" s="16" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="F35" s="16"/>
     </row>
     <row r="36" spans="1:6" outlineLevel="1">
       <c r="A36" s="13" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B36" s="39"/>
       <c r="C36" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D36" s="13" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E36" s="13" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="F36" s="13"/>
     </row>
     <row r="37" spans="1:6" outlineLevel="1">
       <c r="A37" s="16" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B37" s="42"/>
       <c r="C37" s="16" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D37" s="16" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E37" s="16" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="F37" s="16"/>
     </row>
     <row r="38" spans="1:6" outlineLevel="1">
       <c r="A38" s="13" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B38" s="46"/>
       <c r="C38" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D38" s="13" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E38" s="13" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="F38" s="13"/>
     </row>
     <row r="39" spans="1:6" outlineLevel="1">
       <c r="A39" s="16" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B39" s="42"/>
       <c r="C39" s="16" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D39" s="16" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E39" s="16" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="F39" s="16"/>
     </row>
     <row r="40" spans="1:6" outlineLevel="1">
       <c r="A40" s="13" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B40" s="45"/>
       <c r="C40" s="13" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D40" s="13" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E40" s="13" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="F40" s="13"/>
     </row>
     <row r="41" spans="1:6" outlineLevel="1">
       <c r="A41" s="16" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B41" s="47"/>
       <c r="C41" s="16" t="s">
+        <v>84</v>
+      </c>
+      <c r="D41" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="E41" s="16" t="s">
         <v>85</v>
-      </c>
-      <c r="D41" s="16" t="s">
-        <v>51</v>
-      </c>
-      <c r="E41" s="16" t="s">
-        <v>86</v>
       </c>
       <c r="F41" s="16"/>
     </row>
     <row r="42" spans="1:6" outlineLevel="1">
       <c r="A42" s="13" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B42" s="39"/>
       <c r="C42" s="13" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D42" s="13" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E42" s="13" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="F42" s="13"/>
     </row>
     <row r="43" spans="1:6">
       <c r="A43" s="31" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B43" s="43"/>
       <c r="C43" s="15"/>
       <c r="D43" s="15"/>
-      <c r="E43" s="15" t="s">
-        <v>11</v>
-      </c>
+      <c r="E43" s="15"/>
       <c r="F43" s="15"/>
     </row>
     <row r="44" spans="1:6" outlineLevel="1">
       <c r="A44" s="13" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B44" s="39"/>
       <c r="C44" s="13" t="s">
         <v>9</v>
       </c>
       <c r="D44" s="13" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E44" s="13" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="F44" s="13"/>
     </row>
     <row r="45" spans="1:6" outlineLevel="1">
       <c r="A45" s="16" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B45" s="42"/>
       <c r="C45" s="16" t="s">
         <v>9</v>
       </c>
       <c r="D45" s="16" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E45" s="16" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="F45" s="16"/>
     </row>
     <row r="46" spans="1:6" outlineLevel="1">
       <c r="A46" s="13" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B46" s="39"/>
       <c r="C46" s="13" t="s">
         <v>9</v>
       </c>
       <c r="D46" s="13" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E46" s="13" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="F46" s="13"/>
     </row>
     <row r="47" spans="1:6" outlineLevel="1">
       <c r="A47" s="16" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B47" s="42"/>
       <c r="C47" s="16" t="s">
         <v>9</v>
       </c>
       <c r="D47" s="16" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E47" s="16" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="F47" s="16"/>
     </row>
     <row r="48" spans="1:6" outlineLevel="1">
       <c r="A48" s="13" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B48" s="39"/>
       <c r="C48" s="13" t="s">
         <v>9</v>
       </c>
       <c r="D48" s="13" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E48" s="13" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="F48" s="13"/>
     </row>
     <row r="49" spans="1:6" outlineLevel="1">
       <c r="A49" s="16" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B49" s="42"/>
       <c r="C49" s="16" t="s">
         <v>9</v>
       </c>
       <c r="D49" s="16" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E49" s="16" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="F49" s="16"/>
     </row>
     <row r="50" spans="1:6" outlineLevel="1">
       <c r="A50" s="13" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B50" s="39"/>
       <c r="C50" s="13" t="s">
         <v>9</v>
       </c>
       <c r="D50" s="13" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E50" s="13" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="F50" s="13"/>
     </row>
     <row r="51" spans="1:6" outlineLevel="1">
       <c r="A51" s="16" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B51" s="42"/>
       <c r="C51" s="16" t="s">
         <v>9</v>
       </c>
       <c r="D51" s="16" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E51" s="16" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="F51" s="16"/>
     </row>
     <row r="52" spans="1:6" outlineLevel="1">
       <c r="A52" s="13" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B52" s="39"/>
       <c r="C52" s="13" t="s">
         <v>9</v>
       </c>
       <c r="D52" s="13" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E52" s="13" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="F52" s="13"/>
     </row>
     <row r="53" spans="1:6" outlineLevel="1">
       <c r="A53" s="16" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B53" s="42"/>
       <c r="C53" s="16" t="s">
         <v>9</v>
       </c>
       <c r="D53" s="16" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E53" s="16" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="F53" s="16"/>
     </row>
     <row r="54" spans="1:6">
       <c r="A54" s="32" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B54" s="48"/>
       <c r="C54" s="17"/>
@@ -3238,7 +3221,7 @@
     </row>
     <row r="55" spans="1:6" outlineLevel="1">
       <c r="A55" s="18" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B55" s="49"/>
       <c r="C55" s="18" t="s">
@@ -3248,29 +3231,29 @@
         <v>10</v>
       </c>
       <c r="E55" s="18" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="F55" s="18"/>
     </row>
     <row r="56" spans="1:6" outlineLevel="1">
       <c r="A56" s="13" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B56" s="39"/>
       <c r="C56" s="13" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D56" s="13" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E56" s="13" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="F56" s="13"/>
     </row>
     <row r="57" spans="1:6" outlineLevel="1">
       <c r="A57" s="18" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B57" s="49"/>
       <c r="C57" s="18" t="s">
@@ -3280,29 +3263,29 @@
         <v>10</v>
       </c>
       <c r="E57" s="18" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="F57" s="18"/>
     </row>
     <row r="58" spans="1:6" outlineLevel="1">
       <c r="A58" s="13" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="B58" s="39"/>
       <c r="C58" s="13" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D58" s="13" t="s">
         <v>10</v>
       </c>
       <c r="E58" s="13" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="F58" s="13"/>
     </row>
     <row r="59" spans="1:6" outlineLevel="1">
       <c r="A59" s="18" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B59" s="49"/>
       <c r="C59" s="18" t="s">
@@ -3312,29 +3295,29 @@
         <v>10</v>
       </c>
       <c r="E59" s="18" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="F59" s="18"/>
     </row>
     <row r="60" spans="1:6" outlineLevel="1">
       <c r="A60" s="13" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B60" s="39"/>
       <c r="C60" s="13" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D60" s="13" t="s">
         <v>10</v>
       </c>
       <c r="E60" s="13" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F60" s="13"/>
     </row>
     <row r="61" spans="1:6" outlineLevel="1">
       <c r="A61" s="18" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B61" s="49"/>
       <c r="C61" s="18" t="s">
@@ -3344,513 +3327,507 @@
         <v>10</v>
       </c>
       <c r="E61" s="18" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="F61" s="18"/>
     </row>
     <row r="62" spans="1:6" outlineLevel="1">
       <c r="A62" s="13" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B62" s="39"/>
       <c r="C62" s="13" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D62" s="13" t="s">
         <v>10</v>
       </c>
       <c r="E62" s="13" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="F62" s="13"/>
     </row>
     <row r="63" spans="1:6" outlineLevel="1">
       <c r="A63" s="18" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B63" s="49"/>
       <c r="C63" s="18" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D63" s="18" t="s">
         <v>10</v>
       </c>
       <c r="E63" s="18" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="F63" s="18"/>
     </row>
     <row r="64" spans="1:6" outlineLevel="1">
       <c r="A64" s="13" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B64" s="39"/>
       <c r="C64" s="13" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D64" s="13" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E64" s="13" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="F64" s="13"/>
     </row>
     <row r="65" spans="1:6">
       <c r="A65" s="33" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="B65" s="50"/>
       <c r="C65" s="19"/>
       <c r="D65" s="19"/>
-      <c r="E65" s="19" t="s">
-        <v>11</v>
-      </c>
+      <c r="E65" s="19"/>
       <c r="F65" s="19"/>
     </row>
     <row r="66" spans="1:6" outlineLevel="1">
       <c r="A66" s="13" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B66" s="39"/>
       <c r="C66" s="13" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D66" s="13" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E66" s="13" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="F66" s="13"/>
     </row>
     <row r="67" spans="1:6" outlineLevel="1">
       <c r="A67" s="18" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B67" s="51"/>
       <c r="C67" s="18" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D67" s="18" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E67" s="18" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="F67" s="18"/>
     </row>
     <row r="68" spans="1:6" outlineLevel="1">
       <c r="A68" s="13" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B68" s="39"/>
       <c r="C68" s="13" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D68" s="13" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E68" s="13" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="F68" s="13"/>
     </row>
     <row r="69" spans="1:6">
       <c r="A69" s="33" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B69" s="50"/>
       <c r="C69" s="19"/>
       <c r="D69" s="19"/>
-      <c r="E69" s="19" t="s">
-        <v>11</v>
-      </c>
+      <c r="E69" s="19"/>
       <c r="F69" s="19"/>
     </row>
     <row r="70" spans="1:6" outlineLevel="1">
       <c r="A70" s="13" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="B70" s="39"/>
       <c r="C70" s="13" t="s">
         <v>9</v>
       </c>
       <c r="D70" s="13" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E70" s="13" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="F70" s="13"/>
     </row>
     <row r="71" spans="1:6" outlineLevel="1">
       <c r="A71" s="18" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B71" s="52"/>
       <c r="C71" s="18" t="s">
         <v>9</v>
       </c>
       <c r="D71" s="18" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E71" s="18" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="F71" s="18"/>
     </row>
     <row r="72" spans="1:6" outlineLevel="1">
       <c r="A72" s="13" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B72" s="46"/>
       <c r="C72" s="13" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D72" s="13" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E72" s="13" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="F72" s="13"/>
     </row>
     <row r="73" spans="1:6" outlineLevel="1">
       <c r="A73" s="18" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B73" s="53"/>
       <c r="C73" s="18" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D73" s="18" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E73" s="18" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="F73" s="18"/>
     </row>
     <row r="74" spans="1:6" outlineLevel="1">
       <c r="A74" s="13" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B74" s="39"/>
       <c r="C74" s="13" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D74" s="13" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E74" s="13" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="F74" s="13"/>
     </row>
     <row r="75" spans="1:6" outlineLevel="1">
       <c r="A75" s="18" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B75" s="53"/>
       <c r="C75" s="18" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D75" s="18" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E75" s="18" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="F75" s="18"/>
     </row>
     <row r="76" spans="1:6" outlineLevel="1">
       <c r="A76" s="13" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B76" s="39"/>
       <c r="C76" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D76" s="13" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E76" s="13" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="F76" s="13"/>
     </row>
     <row r="77" spans="1:6" outlineLevel="1">
       <c r="A77" s="18" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B77" s="53"/>
       <c r="C77" s="18" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D77" s="18" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E77" s="18" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="F77" s="18"/>
     </row>
     <row r="78" spans="1:6" outlineLevel="1">
       <c r="A78" s="13" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B78" s="46"/>
       <c r="C78" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D78" s="13" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E78" s="13" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="F78" s="13"/>
     </row>
     <row r="79" spans="1:6" outlineLevel="1">
       <c r="A79" s="18" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B79" s="53"/>
       <c r="C79" s="18" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D79" s="18" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E79" s="18" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="F79" s="18"/>
     </row>
     <row r="80" spans="1:6" outlineLevel="1">
       <c r="A80" s="13" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B80" s="46"/>
       <c r="C80" s="13" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D80" s="13" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E80" s="13" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="F80" s="13"/>
     </row>
     <row r="81" spans="1:6" outlineLevel="1">
       <c r="A81" s="18" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="B81" s="54"/>
       <c r="C81" s="18" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D81" s="18" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E81" s="18" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="F81" s="18"/>
     </row>
     <row r="82" spans="1:6" outlineLevel="1">
       <c r="A82" s="13" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="B82" s="55"/>
       <c r="C82" s="13" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D82" s="13" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E82" s="13" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="F82" s="13"/>
     </row>
     <row r="83" spans="1:6">
       <c r="A83" s="33" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="B83" s="50"/>
       <c r="C83" s="19"/>
       <c r="D83" s="19"/>
-      <c r="E83" s="19" t="s">
-        <v>11</v>
-      </c>
+      <c r="E83" s="19"/>
       <c r="F83" s="19"/>
     </row>
     <row r="84" spans="1:6" outlineLevel="1">
       <c r="A84" s="13" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="B84" s="39"/>
       <c r="C84" s="13" t="s">
         <v>9</v>
       </c>
       <c r="D84" s="13" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E84" s="13" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="F84" s="13"/>
     </row>
     <row r="85" spans="1:6" outlineLevel="1">
       <c r="A85" s="18" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="B85" s="49"/>
       <c r="C85" s="18" t="s">
         <v>9</v>
       </c>
       <c r="D85" s="18" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E85" s="18" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="F85" s="18"/>
     </row>
     <row r="86" spans="1:6" outlineLevel="1">
       <c r="A86" s="13" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B86" s="39"/>
       <c r="C86" s="13" t="s">
         <v>9</v>
       </c>
       <c r="D86" s="13" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E86" s="13" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="F86" s="13"/>
     </row>
     <row r="87" spans="1:6" outlineLevel="1">
       <c r="A87" s="18" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B87" s="49"/>
       <c r="C87" s="18" t="s">
         <v>9</v>
       </c>
       <c r="D87" s="18" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E87" s="18" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="F87" s="18"/>
     </row>
     <row r="88" spans="1:6" outlineLevel="1">
       <c r="A88" s="13" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="B88" s="39"/>
       <c r="C88" s="13" t="s">
         <v>9</v>
       </c>
       <c r="D88" s="13" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E88" s="13" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="F88" s="13"/>
     </row>
     <row r="89" spans="1:6" outlineLevel="1">
       <c r="A89" s="18" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="B89" s="49"/>
       <c r="C89" s="18" t="s">
         <v>9</v>
       </c>
       <c r="D89" s="18" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E89" s="18" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="F89" s="18"/>
     </row>
     <row r="90" spans="1:6" outlineLevel="1">
       <c r="A90" s="13" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="B90" s="39"/>
       <c r="C90" s="13" t="s">
         <v>9</v>
       </c>
       <c r="D90" s="13" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E90" s="13" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="F90" s="13"/>
     </row>
     <row r="91" spans="1:6" outlineLevel="1">
       <c r="A91" s="18" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="B91" s="49"/>
       <c r="C91" s="18" t="s">
         <v>9</v>
       </c>
       <c r="D91" s="18" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E91" s="18" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="F91" s="18"/>
     </row>
     <row r="92" spans="1:6" outlineLevel="1">
       <c r="A92" s="13" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="B92" s="39"/>
       <c r="C92" s="13" t="s">
         <v>9</v>
       </c>
       <c r="D92" s="13" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E92" s="13" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="F92" s="13"/>
     </row>
     <row r="93" spans="1:6" outlineLevel="1">
       <c r="A93" s="18" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="B93" s="49"/>
       <c r="C93" s="18" t="s">
         <v>9</v>
       </c>
       <c r="D93" s="18" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E93" s="18" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="F93" s="18"/>
     </row>
     <row r="94" spans="1:6">
       <c r="A94" s="34" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="B94" s="56"/>
       <c r="C94" s="20"/>
@@ -3860,7 +3837,7 @@
     </row>
     <row r="95" spans="1:6" outlineLevel="1">
       <c r="A95" s="13" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="B95" s="39"/>
       <c r="C95" s="13" t="s">
@@ -3870,61 +3847,61 @@
         <v>10</v>
       </c>
       <c r="E95" s="13" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="F95" s="13"/>
     </row>
     <row r="96" spans="1:6" outlineLevel="1">
       <c r="A96" s="21" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="B96" s="57"/>
       <c r="C96" s="21" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D96" s="21" t="s">
         <v>10</v>
       </c>
       <c r="E96" s="21" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="F96" s="21"/>
     </row>
     <row r="97" spans="1:6" outlineLevel="1">
       <c r="A97" s="13" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="B97" s="39"/>
       <c r="C97" s="13" t="s">
         <v>9</v>
       </c>
       <c r="D97" s="13" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E97" s="13" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="F97" s="13"/>
     </row>
     <row r="98" spans="1:6" outlineLevel="1">
       <c r="A98" s="21" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="B98" s="57"/>
       <c r="C98" s="21" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D98" s="22" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E98" s="21" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="F98" s="21"/>
     </row>
     <row r="99" spans="1:6" outlineLevel="1">
       <c r="A99" s="13" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="B99" s="39"/>
       <c r="C99" s="13" t="s">
@@ -3934,437 +3911,433 @@
         <v>10</v>
       </c>
       <c r="E99" s="13" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="F99" s="13"/>
     </row>
     <row r="100" spans="1:6" outlineLevel="1">
       <c r="A100" s="21" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="B100" s="57"/>
       <c r="C100" s="21" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="D100" s="21" t="s">
         <v>10</v>
       </c>
       <c r="E100" s="21" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="F100" s="21"/>
     </row>
     <row r="101" spans="1:6" outlineLevel="1">
       <c r="A101" s="13" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="B101" s="39"/>
       <c r="C101" s="13" t="s">
         <v>9</v>
       </c>
       <c r="D101" s="13" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E101" s="13" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="F101" s="13"/>
     </row>
     <row r="102" spans="1:6" outlineLevel="1">
       <c r="A102" s="21" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B102" s="57"/>
       <c r="C102" s="21" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="D102" s="21" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E102" s="21" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="F102" s="21"/>
     </row>
     <row r="103" spans="1:6" outlineLevel="1">
       <c r="A103" s="13" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="B103" s="39"/>
       <c r="C103" s="13" t="s">
         <v>9</v>
       </c>
       <c r="D103" s="13" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E103" s="13" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="F103" s="13"/>
     </row>
     <row r="104" spans="1:6" outlineLevel="1">
       <c r="A104" s="21" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="B104" s="57"/>
       <c r="C104" s="21" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="D104" s="21" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E104" s="21" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="F104" s="21"/>
     </row>
     <row r="105" spans="1:6" outlineLevel="1">
       <c r="A105" s="13" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="B105" s="39"/>
       <c r="C105" s="13" t="s">
         <v>9</v>
       </c>
       <c r="D105" s="13" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E105" s="13" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="F105" s="13"/>
     </row>
     <row r="106" spans="1:6" outlineLevel="1">
       <c r="A106" s="21" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B106" s="57"/>
       <c r="C106" s="21" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="D106" s="21" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E106" s="21" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="F106" s="21"/>
     </row>
     <row r="107" spans="1:6">
       <c r="A107" s="35" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B107" s="58"/>
       <c r="C107" s="20"/>
       <c r="D107" s="20"/>
-      <c r="E107" s="20" t="s">
-        <v>11</v>
-      </c>
+      <c r="E107" s="20"/>
       <c r="F107" s="20"/>
     </row>
     <row r="108" spans="1:6" outlineLevel="1">
       <c r="A108" s="21" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B108" s="57"/>
       <c r="C108" s="21" t="s">
+        <v>197</v>
+      </c>
+      <c r="D108" s="21" t="s">
+        <v>50</v>
+      </c>
+      <c r="E108" s="21" t="s">
         <v>198</v>
-      </c>
-      <c r="D108" s="21" t="s">
-        <v>51</v>
-      </c>
-      <c r="E108" s="21" t="s">
-        <v>199</v>
       </c>
       <c r="F108" s="21"/>
     </row>
     <row r="109" spans="1:6" outlineLevel="1">
       <c r="A109" s="13" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="B109" s="59"/>
       <c r="C109" s="13" t="s">
+        <v>200</v>
+      </c>
+      <c r="D109" s="13" t="s">
+        <v>50</v>
+      </c>
+      <c r="E109" s="13" t="s">
         <v>201</v>
-      </c>
-      <c r="D109" s="13" t="s">
-        <v>51</v>
-      </c>
-      <c r="E109" s="13" t="s">
-        <v>202</v>
       </c>
       <c r="F109" s="13"/>
     </row>
     <row r="110" spans="1:6" outlineLevel="1">
       <c r="A110" s="21" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="B110" s="57"/>
       <c r="C110" s="21" t="s">
+        <v>203</v>
+      </c>
+      <c r="D110" s="21" t="s">
+        <v>50</v>
+      </c>
+      <c r="E110" s="21" t="s">
         <v>204</v>
-      </c>
-      <c r="D110" s="21" t="s">
-        <v>51</v>
-      </c>
-      <c r="E110" s="21" t="s">
-        <v>205</v>
       </c>
       <c r="F110" s="21"/>
     </row>
     <row r="111" spans="1:6" outlineLevel="1">
       <c r="A111" s="13" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="B111" s="59"/>
       <c r="C111" s="13" t="s">
+        <v>206</v>
+      </c>
+      <c r="D111" s="13" t="s">
+        <v>50</v>
+      </c>
+      <c r="E111" s="23" t="s">
         <v>207</v>
-      </c>
-      <c r="D111" s="13" t="s">
-        <v>51</v>
-      </c>
-      <c r="E111" s="23" t="s">
-        <v>208</v>
       </c>
       <c r="F111" s="13"/>
     </row>
     <row r="112" spans="1:6">
       <c r="A112" s="35" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="B112" s="58"/>
       <c r="C112" s="20"/>
       <c r="D112" s="20"/>
-      <c r="E112" s="20" t="s">
-        <v>11</v>
-      </c>
+      <c r="E112" s="20"/>
       <c r="F112" s="20"/>
     </row>
     <row r="113" spans="1:6" outlineLevel="1">
       <c r="A113" s="13" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B113" s="39"/>
       <c r="C113" s="13" t="s">
         <v>9</v>
       </c>
       <c r="D113" s="13" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E113" s="13" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="F113" s="13"/>
     </row>
     <row r="114" spans="1:6" outlineLevel="1">
       <c r="A114" s="21" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="B114" s="57"/>
       <c r="C114" s="21" t="s">
         <v>9</v>
       </c>
       <c r="D114" s="21" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E114" s="21" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="F114" s="21"/>
     </row>
     <row r="115" spans="1:6" outlineLevel="1">
       <c r="A115" s="13" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="B115" s="39"/>
       <c r="C115" s="13" t="s">
         <v>9</v>
       </c>
       <c r="D115" s="13" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E115" s="13" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="F115" s="13"/>
     </row>
     <row r="116" spans="1:6" outlineLevel="1">
       <c r="A116" s="21" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="B116" s="57"/>
       <c r="C116" s="21" t="s">
         <v>9</v>
       </c>
       <c r="D116" s="21" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E116" s="21" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="F116" s="21"/>
     </row>
     <row r="117" spans="1:6" outlineLevel="1">
       <c r="A117" s="13" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="B117" s="39"/>
       <c r="C117" s="13" t="s">
         <v>9</v>
       </c>
       <c r="D117" s="13" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E117" s="13" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="F117" s="13"/>
     </row>
     <row r="118" spans="1:6" outlineLevel="1">
       <c r="A118" s="24" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="B118" s="60"/>
       <c r="C118" s="24" t="s">
         <v>9</v>
       </c>
       <c r="D118" s="24" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E118" s="24" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="F118" s="21"/>
     </row>
     <row r="119" spans="1:6" outlineLevel="1" collapsed="1">
       <c r="A119" s="13" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="B119" s="55"/>
       <c r="C119" s="13" t="s">
         <v>9</v>
       </c>
       <c r="D119" s="13" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E119" s="13" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="F119" s="13"/>
     </row>
     <row r="120" spans="1:6" outlineLevel="1">
       <c r="A120" s="21" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="B120" s="57"/>
       <c r="C120" s="21" t="s">
         <v>9</v>
       </c>
       <c r="D120" s="21" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E120" s="21" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="F120" s="21"/>
     </row>
     <row r="121" spans="1:6" outlineLevel="1">
       <c r="A121" s="13" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="B121" s="39"/>
       <c r="C121" s="13" t="s">
         <v>9</v>
       </c>
       <c r="D121" s="13" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E121" s="13" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="F121" s="13"/>
     </row>
     <row r="122" spans="1:6" outlineLevel="1" collapsed="1">
       <c r="A122" s="21" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="B122" s="57"/>
       <c r="C122" s="21" t="s">
         <v>9</v>
       </c>
       <c r="D122" s="21" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E122" s="21" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="F122" s="21"/>
     </row>
     <row r="123" spans="1:6" outlineLevel="1">
       <c r="A123" s="23" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="B123" s="61"/>
       <c r="C123" s="23" t="s">
         <v>9</v>
       </c>
       <c r="D123" s="23" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E123" s="23" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="F123" s="23"/>
     </row>
     <row r="124" spans="1:6" outlineLevel="1">
       <c r="A124" s="21" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="B124" s="57"/>
       <c r="C124" s="21" t="s">
         <v>9</v>
       </c>
       <c r="D124" s="21" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E124" s="21" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="F124" s="21"/>
     </row>
     <row r="125" spans="1:6" outlineLevel="1">
       <c r="A125" s="23" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="B125" s="61"/>
       <c r="C125" s="23" t="s">
         <v>9</v>
       </c>
       <c r="D125" s="23" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E125" s="23" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="F125" s="23"/>
     </row>
     <row r="126" spans="1:6" outlineLevel="1">
       <c r="A126" s="21" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="B126" s="57"/>
       <c r="C126" s="21" t="s">
         <v>9</v>
       </c>
       <c r="D126" s="21" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E126" s="21" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="F126" s="21"/>
     </row>
     <row r="127" spans="1:6" ht="14.45" customHeight="1">
       <c r="A127" s="36" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="B127" s="62"/>
       <c r="C127" s="25"/>
@@ -4374,7 +4347,7 @@
     </row>
     <row r="128" spans="1:6" outlineLevel="1">
       <c r="A128" s="14" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="B128" s="40"/>
       <c r="C128" s="14" t="s">
@@ -4384,118 +4357,114 @@
         <v>10</v>
       </c>
       <c r="E128" s="14" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="F128" s="14"/>
     </row>
     <row r="129" spans="1:8" outlineLevel="1">
       <c r="A129" s="13" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="B129" s="39"/>
       <c r="C129" s="13" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D129" s="13" t="s">
         <v>10</v>
       </c>
       <c r="E129" s="13" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="F129" s="13"/>
     </row>
     <row r="130" spans="1:8">
       <c r="A130" s="37" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="B130" s="63"/>
       <c r="C130" s="26"/>
       <c r="D130" s="26"/>
-      <c r="E130" s="26" t="s">
-        <v>11</v>
-      </c>
+      <c r="E130" s="26"/>
       <c r="F130" s="26"/>
     </row>
     <row r="131" spans="1:8" outlineLevel="1">
       <c r="A131" s="14" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="B131" s="40"/>
       <c r="C131" s="14" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D131" s="14" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E131" s="14" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="F131" s="14"/>
     </row>
     <row r="132" spans="1:8" outlineLevel="1">
       <c r="A132" s="13" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="B132" s="39"/>
       <c r="C132" s="13" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D132" s="13" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E132" s="13" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="F132" s="23"/>
       <c r="H132" s="12"/>
     </row>
     <row r="133" spans="1:8">
       <c r="A133" s="37" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="B133" s="63"/>
       <c r="C133" s="26"/>
       <c r="D133" s="26"/>
-      <c r="E133" s="26" t="s">
-        <v>11</v>
-      </c>
+      <c r="E133" s="26"/>
       <c r="F133" s="26"/>
     </row>
     <row r="134" spans="1:8" outlineLevel="1">
       <c r="A134" s="13" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="B134" s="39"/>
       <c r="C134" s="13" t="s">
         <v>9</v>
       </c>
       <c r="D134" s="13" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E134" s="13" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="F134" s="23"/>
     </row>
     <row r="135" spans="1:8" outlineLevel="1">
       <c r="A135" s="14" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="B135" s="40"/>
       <c r="C135" s="14" t="s">
         <v>9</v>
       </c>
       <c r="D135" s="14" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E135" s="14" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="F135" s="14"/>
     </row>
     <row r="136" spans="1:8">
       <c r="A136" s="36" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="B136" s="62"/>
       <c r="C136" s="25"/>
@@ -4505,7 +4474,7 @@
     </row>
     <row r="137" spans="1:8" outlineLevel="1">
       <c r="A137" s="14" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="B137" s="40"/>
       <c r="C137" s="14" t="s">
@@ -4515,13 +4484,13 @@
         <v>10</v>
       </c>
       <c r="E137" s="14" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="F137" s="14"/>
     </row>
     <row r="138" spans="1:8" outlineLevel="1">
       <c r="A138" s="13" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="B138" s="39"/>
       <c r="C138" s="13" t="s">
@@ -4531,13 +4500,13 @@
         <v>10</v>
       </c>
       <c r="E138" s="13" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="F138" s="13"/>
     </row>
     <row r="139" spans="1:8" outlineLevel="1">
       <c r="A139" s="14" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="B139" s="40"/>
       <c r="C139" s="14" t="s">
@@ -4547,13 +4516,13 @@
         <v>10</v>
       </c>
       <c r="E139" s="14" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="F139" s="14"/>
     </row>
     <row r="140" spans="1:8" outlineLevel="1">
       <c r="A140" s="13" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="B140" s="39"/>
       <c r="C140" s="13" t="s">
@@ -4563,157 +4532,157 @@
         <v>10</v>
       </c>
       <c r="E140" s="13" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="F140" s="13"/>
     </row>
     <row r="141" spans="1:8" outlineLevel="1">
       <c r="A141" s="14" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="B141" s="40"/>
       <c r="C141" s="14" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="D141" s="14" t="s">
         <v>10</v>
       </c>
       <c r="E141" s="14" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="F141" s="14"/>
     </row>
     <row r="142" spans="1:8" outlineLevel="1">
       <c r="A142" s="13" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="B142" s="39"/>
       <c r="C142" s="13" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="D142" s="13" t="s">
         <v>10</v>
       </c>
       <c r="E142" s="13" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="F142" s="13"/>
     </row>
     <row r="143" spans="1:8" outlineLevel="1">
       <c r="A143" s="14" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="B143" s="40"/>
       <c r="C143" s="14" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="D143" s="14" t="s">
         <v>10</v>
       </c>
       <c r="E143" s="27" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="F143" s="14"/>
     </row>
     <row r="144" spans="1:8" outlineLevel="1">
       <c r="A144" s="13" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="B144" s="39"/>
       <c r="C144" s="13" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="D144" s="13" t="s">
         <v>10</v>
       </c>
       <c r="E144" s="13" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="F144" s="13"/>
     </row>
     <row r="145" spans="1:6" outlineLevel="1">
       <c r="A145" s="14" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="B145" s="40"/>
       <c r="C145" s="14" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="D145" s="14" t="s">
         <v>10</v>
       </c>
       <c r="E145" s="14" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="F145" s="14"/>
     </row>
     <row r="146" spans="1:6" outlineLevel="1">
       <c r="A146" s="13" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="B146" s="39"/>
       <c r="C146" s="13" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="D146" s="13" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E146" s="13" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="F146" s="13"/>
     </row>
     <row r="147" spans="1:6" outlineLevel="1">
       <c r="A147" s="14" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="B147" s="40"/>
       <c r="C147" s="14" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="D147" s="14" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E147" s="14" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="F147" s="14"/>
     </row>
     <row r="148" spans="1:6" outlineLevel="1">
       <c r="A148" s="13" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="B148" s="39"/>
       <c r="C148" s="13" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="D148" s="13" t="s">
         <v>10</v>
       </c>
       <c r="E148" s="13" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="F148" s="13"/>
     </row>
     <row r="149" spans="1:6" outlineLevel="1">
       <c r="A149" s="14" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="B149" s="40"/>
       <c r="C149" s="14" t="s">
         <v>9</v>
       </c>
       <c r="D149" s="14" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E149" s="14" t="s">
-        <v>5</v>
+        <v>404</v>
       </c>
       <c r="F149" s="14"/>
     </row>
     <row r="150" spans="1:6">
       <c r="A150" s="37" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="B150" s="64"/>
       <c r="C150" s="26"/>
@@ -4723,33 +4692,33 @@
     </row>
     <row r="151" spans="1:6" outlineLevel="1">
       <c r="A151" s="13" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="B151" s="39"/>
       <c r="C151" s="13" t="s">
         <v>9</v>
       </c>
       <c r="D151" s="13" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E151" s="13" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="F151" s="13"/>
     </row>
     <row r="152" spans="1:6" outlineLevel="1">
       <c r="A152" s="14" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="B152" s="40"/>
       <c r="C152" s="14" t="s">
         <v>9</v>
       </c>
       <c r="D152" s="14" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E152" s="14" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="F152" s="14"/>
     </row>
@@ -4808,11 +4777,11 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D34">
-    <cfRule type="expression" dxfId="24" priority="22">
+    <cfRule type="expression" dxfId="24" priority="23">
+      <formula>$B29="Hide"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="23" priority="22">
       <formula>#REF!="Hide"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="23" priority="23">
-      <formula>$B29="Hide"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D38">
@@ -4871,11 +4840,11 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D80">
-    <cfRule type="expression" dxfId="11" priority="11">
+    <cfRule type="expression" dxfId="11" priority="12">
+      <formula>$B78="Hide"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="10" priority="11">
       <formula>$B76="Hide"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="10" priority="12">
-      <formula>$B78="Hide"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D81">
@@ -4939,66 +4908,66 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="6" t="s">
+        <v>264</v>
+      </c>
+      <c r="B1" s="6" t="s">
         <v>265</v>
-      </c>
-      <c r="B1" s="6" t="s">
-        <v>266</v>
       </c>
     </row>
     <row r="2" spans="1:2">
       <c r="A2" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
     </row>
     <row r="3" spans="1:2">
       <c r="A3" t="s">
+        <v>267</v>
+      </c>
+      <c r="B3" s="1" t="s">
         <v>268</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>269</v>
       </c>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" t="s">
+        <v>269</v>
+      </c>
+      <c r="B4" s="1" t="s">
         <v>270</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>271</v>
       </c>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" t="s">
+        <v>271</v>
+      </c>
+      <c r="B5" s="1" t="s">
         <v>272</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>273</v>
       </c>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" t="s">
+        <v>274</v>
+      </c>
+      <c r="B7" s="1" t="s">
         <v>275</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>276</v>
       </c>
     </row>
     <row r="8" spans="1:2">
       <c r="A8" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
     </row>
   </sheetData>
@@ -5025,145 +4994,145 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="11" t="s">
+        <v>264</v>
+      </c>
+      <c r="B1" s="11" t="s">
         <v>265</v>
-      </c>
-      <c r="B1" s="11" t="s">
-        <v>266</v>
       </c>
     </row>
     <row r="2" spans="1:2">
       <c r="A2" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="3" spans="1:2">
       <c r="A3" t="s">
+        <v>278</v>
+      </c>
+      <c r="B3" t="s">
         <v>279</v>
-      </c>
-      <c r="B3" t="s">
-        <v>280</v>
       </c>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" t="s">
+        <v>281</v>
+      </c>
+      <c r="B6" t="s">
         <v>282</v>
-      </c>
-      <c r="B6" t="s">
-        <v>283</v>
       </c>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" t="s">
+        <v>283</v>
+      </c>
+      <c r="B7" t="s">
         <v>284</v>
-      </c>
-      <c r="B7" t="s">
-        <v>285</v>
       </c>
     </row>
     <row r="8" spans="1:2">
       <c r="A8" t="s">
+        <v>285</v>
+      </c>
+      <c r="B8" t="s">
         <v>286</v>
-      </c>
-      <c r="B8" t="s">
-        <v>287</v>
       </c>
     </row>
     <row r="9" spans="1:2">
       <c r="A9" t="s">
+        <v>287</v>
+      </c>
+      <c r="B9" t="s">
         <v>288</v>
-      </c>
-      <c r="B9" t="s">
-        <v>289</v>
       </c>
     </row>
     <row r="10" spans="1:2">
       <c r="A10" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="B10" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="11" spans="1:2">
       <c r="A11" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="B11" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
     </row>
     <row r="12" spans="1:2">
       <c r="A12" t="s">
+        <v>290</v>
+      </c>
+      <c r="B12" t="s">
         <v>291</v>
-      </c>
-      <c r="B12" t="s">
-        <v>292</v>
       </c>
     </row>
     <row r="13" spans="1:2">
       <c r="A13" t="s">
+        <v>292</v>
+      </c>
+      <c r="B13" t="s">
         <v>293</v>
-      </c>
-      <c r="B13" t="s">
-        <v>294</v>
       </c>
     </row>
     <row r="14" spans="1:2">
       <c r="A14" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="B14" s="7"/>
     </row>
     <row r="15" spans="1:2">
       <c r="A15" s="2" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="B15" s="8"/>
     </row>
     <row r="16" spans="1:2">
       <c r="A16" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
     </row>
     <row r="17" spans="1:2">
       <c r="A17" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
     </row>
     <row r="18" spans="1:2">
       <c r="A18" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
     </row>
     <row r="19" spans="1:2">
       <c r="A19" t="s">
+        <v>299</v>
+      </c>
+      <c r="B19" t="s">
         <v>300</v>
-      </c>
-      <c r="B19" t="s">
-        <v>301</v>
       </c>
     </row>
     <row r="20" spans="1:2">
       <c r="A20" t="s">
+        <v>302</v>
+      </c>
+      <c r="B20" t="s">
         <v>303</v>
-      </c>
-      <c r="B20" t="s">
-        <v>304</v>
       </c>
     </row>
     <row r="21" spans="1:2">
       <c r="A21" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
     </row>
   </sheetData>
@@ -5189,206 +5158,206 @@
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" s="6" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="B1" s="6" t="s">
+        <v>326</v>
+      </c>
+      <c r="C1" s="6" t="s">
         <v>327</v>
-      </c>
-      <c r="C1" s="6" t="s">
-        <v>328</v>
       </c>
     </row>
     <row r="2" spans="1:3">
       <c r="A2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C2" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
     </row>
     <row r="3" spans="1:3">
       <c r="A3" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="4" spans="1:3">
       <c r="A4" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="C4" s="10" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
     </row>
     <row r="5" spans="1:3">
       <c r="A5" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="6" spans="1:3">
       <c r="A6" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="7" spans="1:3">
       <c r="A7" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="8" spans="1:3">
       <c r="A8" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="9" spans="1:3">
       <c r="A9" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
     </row>
     <row r="10" spans="1:3">
       <c r="A10" s="5" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
     </row>
     <row r="11" spans="1:3">
       <c r="A11" s="5" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
     </row>
     <row r="12" spans="1:3">
       <c r="A12" s="5" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
     </row>
     <row r="13" spans="1:3">
       <c r="A13" s="5" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
     </row>
     <row r="14" spans="1:3">
       <c r="A14" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
     </row>
     <row r="15" spans="1:3">
       <c r="A15" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
     </row>
     <row r="16" spans="1:3">
       <c r="A16" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B16" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
     </row>
     <row r="17" spans="1:2">
       <c r="A17" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="B17" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
     </row>
     <row r="18" spans="1:2">
       <c r="A18" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="B18" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
     </row>
     <row r="19" spans="1:2">
       <c r="A19" t="s">
+        <v>390</v>
+      </c>
+      <c r="B19" t="s">
         <v>391</v>
-      </c>
-      <c r="B19" t="s">
-        <v>392</v>
       </c>
     </row>
     <row r="20" spans="1:2">
       <c r="A20" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B20" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
     </row>
     <row r="21" spans="1:2">
       <c r="A21" t="s">
+        <v>336</v>
+      </c>
+      <c r="B21" s="10" t="s">
         <v>337</v>
-      </c>
-      <c r="B21" s="10" t="s">
-        <v>338</v>
       </c>
     </row>
     <row r="22" spans="1:2">
       <c r="A22" t="s">
+        <v>338</v>
+      </c>
+      <c r="B22" t="s">
         <v>339</v>
-      </c>
-      <c r="B22" t="s">
-        <v>340</v>
       </c>
     </row>
     <row r="23" spans="1:2">
       <c r="A23" t="s">
+        <v>340</v>
+      </c>
+      <c r="B23" t="s">
         <v>341</v>
-      </c>
-      <c r="B23" t="s">
-        <v>342</v>
       </c>
     </row>
     <row r="24" spans="1:2">
       <c r="A24" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
     <row r="25" spans="1:2">
       <c r="A25" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
     </row>
     <row r="26" spans="1:2">
       <c r="A26" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="27" spans="1:2">
       <c r="A27" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
     </row>
     <row r="28" spans="1:2">
       <c r="A28" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="29" spans="1:2">
       <c r="A29" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="30" spans="1:2">
       <c r="A30" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
     </row>
     <row r="31" spans="1:2">
       <c r="A31" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
     </row>
     <row r="32" spans="1:2">
       <c r="A32" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
     </row>
     <row r="33" spans="1:1">
       <c r="A33" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
     </row>
   </sheetData>
@@ -5411,154 +5380,154 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="6" t="s">
+        <v>264</v>
+      </c>
+      <c r="B1" s="6" t="s">
         <v>265</v>
-      </c>
-      <c r="B1" s="6" t="s">
-        <v>266</v>
       </c>
     </row>
     <row r="2" spans="1:2">
       <c r="A2" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="B2" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
     </row>
     <row r="3" spans="1:2">
       <c r="A3" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B3" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B4" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" t="s">
+        <v>307</v>
+      </c>
+      <c r="B5" s="3" t="s">
         <v>308</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>309</v>
       </c>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" t="s">
+        <v>309</v>
+      </c>
+      <c r="B6" s="3" t="s">
         <v>310</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>311</v>
       </c>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B7" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
     </row>
     <row r="8" spans="1:2">
       <c r="A8" t="s">
+        <v>312</v>
+      </c>
+      <c r="B8" t="s">
         <v>313</v>
-      </c>
-      <c r="B8" t="s">
-        <v>314</v>
       </c>
     </row>
     <row r="9" spans="1:2">
       <c r="A9" t="s">
+        <v>314</v>
+      </c>
+      <c r="B9" t="s">
         <v>315</v>
-      </c>
-      <c r="B9" t="s">
-        <v>316</v>
       </c>
     </row>
     <row r="10" spans="1:2">
       <c r="A10" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B10" s="9" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
     </row>
     <row r="11" spans="1:2">
       <c r="A11" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B11" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
     </row>
     <row r="12" spans="1:2">
       <c r="A12" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B12" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
     </row>
     <row r="13" spans="1:2">
       <c r="A13" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B13" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
     </row>
     <row r="14" spans="1:2">
       <c r="A14" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="B14" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
     </row>
     <row r="15" spans="1:2">
       <c r="A15" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B15" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
     </row>
     <row r="16" spans="1:2">
       <c r="A16" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="B16" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
     </row>
     <row r="17" spans="1:2">
       <c r="A17" s="2" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
     </row>
     <row r="18" spans="1:2">
       <c r="A18" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
     </row>
     <row r="19" spans="1:2">
       <c r="A19" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B19" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
     </row>
   </sheetData>
@@ -5576,59 +5545,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <FolderType xmlns="35345429-01ed-4d83-85b9-6cc21878d784" xsi:nil="true"/>
-    <CultureName xmlns="35345429-01ed-4d83-85b9-6cc21878d784" xsi:nil="true"/>
-    <Leaders xmlns="35345429-01ed-4d83-85b9-6cc21878d784">
-      <UserInfo>
-        <DisplayName/>
-        <AccountId xsi:nil="true"/>
-        <AccountType/>
-      </UserInfo>
-    </Leaders>
-    <IsNotebookLocked xmlns="35345429-01ed-4d83-85b9-6cc21878d784" xsi:nil="true"/>
-    <Invited_Members xmlns="35345429-01ed-4d83-85b9-6cc21878d784" xsi:nil="true"/>
-    <Math_Settings xmlns="35345429-01ed-4d83-85b9-6cc21878d784" xsi:nil="true"/>
-    <Self_Registration_Enabled xmlns="35345429-01ed-4d83-85b9-6cc21878d784" xsi:nil="true"/>
-    <Has_Leaders_Only_SectionGroup xmlns="35345429-01ed-4d83-85b9-6cc21878d784" xsi:nil="true"/>
-    <Member_Groups xmlns="35345429-01ed-4d83-85b9-6cc21878d784">
-      <UserInfo>
-        <DisplayName/>
-        <AccountId xsi:nil="true"/>
-        <AccountType/>
-      </UserInfo>
-    </Member_Groups>
-    <Distribution_Groups xmlns="35345429-01ed-4d83-85b9-6cc21878d784" xsi:nil="true"/>
-    <AppVersion xmlns="35345429-01ed-4d83-85b9-6cc21878d784" xsi:nil="true"/>
-    <DefaultSectionNames xmlns="35345429-01ed-4d83-85b9-6cc21878d784" xsi:nil="true"/>
-    <Templates xmlns="35345429-01ed-4d83-85b9-6cc21878d784" xsi:nil="true"/>
-    <NotebookType xmlns="35345429-01ed-4d83-85b9-6cc21878d784" xsi:nil="true"/>
-    <TeamsChannelId xmlns="35345429-01ed-4d83-85b9-6cc21878d784" xsi:nil="true"/>
-    <Invited_Leaders xmlns="35345429-01ed-4d83-85b9-6cc21878d784" xsi:nil="true"/>
-    <Is_Collaboration_Space_Locked xmlns="35345429-01ed-4d83-85b9-6cc21878d784" xsi:nil="true"/>
-    <Teams_Channel_Section_Location xmlns="35345429-01ed-4d83-85b9-6cc21878d784" xsi:nil="true"/>
-    <Members xmlns="35345429-01ed-4d83-85b9-6cc21878d784">
-      <UserInfo>
-        <DisplayName/>
-        <AccountId xsi:nil="true"/>
-        <AccountType/>
-      </UserInfo>
-    </Members>
-    <Owner xmlns="35345429-01ed-4d83-85b9-6cc21878d784">
-      <UserInfo>
-        <DisplayName/>
-        <AccountId xsi:nil="true"/>
-        <AccountType/>
-      </UserInfo>
-    </Owner>
-    <LMS_Mappings xmlns="35345429-01ed-4d83-85b9-6cc21878d784" xsi:nil="true"/>
-    <_activity xmlns="35345429-01ed-4d83-85b9-6cc21878d784" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Dokument" ma:contentTypeID="0x010100F5BD758A7F2BF742ADB9291A93682A9E" ma:contentTypeVersion="31" ma:contentTypeDescription="Ein neues Dokument erstellen." ma:contentTypeScope="" ma:versionID="0517f02299b6dbd064809d9c3f869e8a">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="35345429-01ed-4d83-85b9-6cc21878d784" xmlns:ns4="53f86fb7-11c0-476e-bf8b-57768422e991" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="a7ff6e993c77c55b2c02ebba747ae01b" ns3:_="" ns4:_="">
     <xsd:import namespace="35345429-01ed-4d83-85b9-6cc21878d784"/>
@@ -6025,6 +5941,59 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <FolderType xmlns="35345429-01ed-4d83-85b9-6cc21878d784" xsi:nil="true"/>
+    <CultureName xmlns="35345429-01ed-4d83-85b9-6cc21878d784" xsi:nil="true"/>
+    <Leaders xmlns="35345429-01ed-4d83-85b9-6cc21878d784">
+      <UserInfo>
+        <DisplayName/>
+        <AccountId xsi:nil="true"/>
+        <AccountType/>
+      </UserInfo>
+    </Leaders>
+    <IsNotebookLocked xmlns="35345429-01ed-4d83-85b9-6cc21878d784" xsi:nil="true"/>
+    <Invited_Members xmlns="35345429-01ed-4d83-85b9-6cc21878d784" xsi:nil="true"/>
+    <Math_Settings xmlns="35345429-01ed-4d83-85b9-6cc21878d784" xsi:nil="true"/>
+    <Self_Registration_Enabled xmlns="35345429-01ed-4d83-85b9-6cc21878d784" xsi:nil="true"/>
+    <Has_Leaders_Only_SectionGroup xmlns="35345429-01ed-4d83-85b9-6cc21878d784" xsi:nil="true"/>
+    <Member_Groups xmlns="35345429-01ed-4d83-85b9-6cc21878d784">
+      <UserInfo>
+        <DisplayName/>
+        <AccountId xsi:nil="true"/>
+        <AccountType/>
+      </UserInfo>
+    </Member_Groups>
+    <Distribution_Groups xmlns="35345429-01ed-4d83-85b9-6cc21878d784" xsi:nil="true"/>
+    <AppVersion xmlns="35345429-01ed-4d83-85b9-6cc21878d784" xsi:nil="true"/>
+    <DefaultSectionNames xmlns="35345429-01ed-4d83-85b9-6cc21878d784" xsi:nil="true"/>
+    <Templates xmlns="35345429-01ed-4d83-85b9-6cc21878d784" xsi:nil="true"/>
+    <NotebookType xmlns="35345429-01ed-4d83-85b9-6cc21878d784" xsi:nil="true"/>
+    <TeamsChannelId xmlns="35345429-01ed-4d83-85b9-6cc21878d784" xsi:nil="true"/>
+    <Invited_Leaders xmlns="35345429-01ed-4d83-85b9-6cc21878d784" xsi:nil="true"/>
+    <Is_Collaboration_Space_Locked xmlns="35345429-01ed-4d83-85b9-6cc21878d784" xsi:nil="true"/>
+    <Teams_Channel_Section_Location xmlns="35345429-01ed-4d83-85b9-6cc21878d784" xsi:nil="true"/>
+    <Members xmlns="35345429-01ed-4d83-85b9-6cc21878d784">
+      <UserInfo>
+        <DisplayName/>
+        <AccountId xsi:nil="true"/>
+        <AccountType/>
+      </UserInfo>
+    </Members>
+    <Owner xmlns="35345429-01ed-4d83-85b9-6cc21878d784">
+      <UserInfo>
+        <DisplayName/>
+        <AccountId xsi:nil="true"/>
+        <AccountType/>
+      </UserInfo>
+    </Owner>
+    <LMS_Mappings xmlns="35345429-01ed-4d83-85b9-6cc21878d784" xsi:nil="true"/>
+    <_activity xmlns="35345429-01ed-4d83-85b9-6cc21878d784" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E85C156E-EE0C-426A-92B3-CAF84DB17690}">
   <ds:schemaRefs>
@@ -6034,16 +6003,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B2D89A20-922B-4399-8A99-02ABCC3D1E33}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="35345429-01ed-4d83-85b9-6cc21878d784"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0D716C96-A80E-4732-A5D3-9C77E88EE8CA}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -6060,4 +6019,14 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B2D89A20-922B-4399-8A99-02ABCC3D1E33}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="35345429-01ed-4d83-85b9-6cc21878d784"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>